<commit_message>
Rename boss Jerry → Datto
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MSxiXd6jSsJas8jyd5R32w
</commit_message>
<xml_diff>
--- a/config/blast-track-config.xlsx
+++ b/config/blast-track-config.xlsx
@@ -9083,7 +9083,7 @@
       </c>
       <c r="C44" s="9" t="inlineStr">
         <is>
-          <t>Jerry，侧面向右跑；真人原型需本人同意</t>
+          <t>Datto，侧面向右跑；真人原型需本人同意</t>
         </is>
       </c>
       <c r="D44" s="9" t="inlineStr">
@@ -9945,22 +9945,22 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>3 个 Boss 波每局从 6 位传奇跑者里随机抽：Nox（九命复活）、Aurum（召唤金甲跑者）、Slimo（黏液加速）、Rocco（铁头冲刺）、Chuckles（大笑让装置停工）、Jerry（对常用装置产生抗性）。</t>
+          <t>3 个 Boss 波每局从 6 位传奇跑者里随机抽：Nox（九命复活）、Aurum（召唤金甲跑者）、Slimo（黏液加速）、Rocco（铁头冲刺）、Chuckles（大笑让装置停工）、Datto（对常用装置产生抗性）。</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>3 个 Boss 波每局从 6 位传奇跑者里随机抽：Nox（九命复活）、Aurum（召唤金甲跑者）、Slimo（黏液加速）、Rocco（铁头冲刺）、Chuckles（大笑让装置停工）、Jerry（对常用装置产生抗性）。</t>
+          <t>3 个 Boss 波每局从 6 位传奇跑者里随机抽：Nox（九命复活）、Aurum（召唤金甲跑者）、Slimo（黏液加速）、Rocco（铁头冲刺）、Chuckles（大笑让装置停工）、Datto（对常用装置产生抗性）。</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Each run draws 3 bosses from 6 legendary runners: Nox (nine lives), Aurum (summons golden runners), Slimo (slime boost), Rocco (headstrong dash), Chuckles (laughter jams devices), Jerry (adapts to your most-used device).</t>
+          <t>Each run draws 3 bosses from 6 legendary runners: Nox (nine lives), Aurum (summons golden runners), Slimo (slime boost), Rocco (headstrong dash), Chuckles (laughter jams devices), Datto (adapts to your most-used device).</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>Chaque partie tire 3 boss parmi 6 coureurs légendaires : Nox (neuf vies), Aurum (invoque des coureurs dorés), Slimo (bave accélérante), Rocco (charge tête baissée), Chuckles (son rire bloque les dispositifs), Jerry (s’adapte à ton dispositif favori).</t>
+          <t>Chaque partie tire 3 boss parmi 6 coureurs légendaires : Nox (neuf vies), Aurum (invoque des coureurs dorés), Slimo (bave accélérante), Rocco (charge tête baissée), Chuckles (son rire bloque les dispositifs), Datto (s’adapte à ton dispositif favori).</t>
         </is>
       </c>
     </row>
@@ -24145,7 +24145,7 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Jerry</t>
+          <t>Datto</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">

</xml_diff>

<commit_message>
Add chapter-map button to leave classic mode or a level
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MSxiXd6jSsJas8jyd5R32w
</commit_message>
<xml_diff>
--- a/config/blast-track-config.xlsx
+++ b/config/blast-track-config.xlsx
@@ -10213,7 +10213,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D274"/>
+  <dimension ref="A1:D275"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -16206,8 +16206,30 @@
         </is>
       </c>
     </row>
-    <row r="274">
-      <c r="A274" s="10" t="inlineStr">
+    <row r="273">
+      <c r="A273" s="6" t="inlineStr">
+        <is>
+          <t>再点一次离开（本局进度不保存）</t>
+        </is>
+      </c>
+      <c r="B273" s="8" t="inlineStr">
+        <is>
+          <t>再点一次离开（本局进度不保存）</t>
+        </is>
+      </c>
+      <c r="C273" s="8" t="inlineStr">
+        <is>
+          <t>Tap again to leave (this run is not saved)</t>
+        </is>
+      </c>
+      <c r="D273" s="8" t="inlineStr">
+        <is>
+          <t>Touche encore pour quitter (partie non sauvegardée)</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="10" t="inlineStr">
         <is>
           <t>※ 花括号里的 {n}、{x} 等是占位符，翻译时要原样保留。</t>
         </is>

</xml_diff>

<commit_message>
Can Tosser: skeletal part animation (idle/fire/release) + flying can and hit sprites
Parts rig and generator live in art/can-tosser; default art wired via cfg_build.py;
drawArt falls back to vector art while an animation JSON is loading.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019aYuPSmDStWHRUCSamkHbW
</commit_message>
<xml_diff>
--- a/config/blast-track-config.xlsx
+++ b/config/blast-track-config.xlsx
@@ -7607,10 +7607,18 @@
           <t>P1 样板关</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr"/>
-      <c r="F9" s="8" t="inlineStr"/>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.dart.png</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.dart.json</t>
+        </is>
+      </c>
       <c r="G9" s="7" t="n">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="H9" s="7" t="n">
         <v>50</v>
@@ -10400,13 +10408,21 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E66" s="8" t="inlineStr"/>
-      <c r="F66" s="8" t="inlineStr"/>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.dart.png</t>
+        </is>
+      </c>
+      <c r="F66" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.dart.json</t>
+        </is>
+      </c>
       <c r="G66" s="7" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="H66" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="I66" s="7" t="n">
         <v>0.5</v>

</xml_diff>

<commit_message>
Can Tosser path A (重罐点名) tiers 1-6 live: per-tier tower + projectile sheets, A1/A2 attachment art lookup, per-tower shot art
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019aYuPSmDStWHRUCSamkHbW
</commit_message>
<xml_diff>
--- a/config/blast-track-config.xlsx
+++ b/config/blast-track-config.xlsx
@@ -7145,7 +7145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N82"/>
+  <dimension ref="A1:N90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7618,10 +7618,10 @@
         </is>
       </c>
       <c r="G9" s="7" t="n">
-        <v>46</v>
+        <v>44.6</v>
       </c>
       <c r="H9" s="7" t="n">
-        <v>50</v>
+        <v>46.5</v>
       </c>
       <c r="I9" s="7" t="n">
         <v>0.5</v>
@@ -7958,13 +7958,21 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E16" s="8" t="inlineStr"/>
-      <c r="F16" s="8" t="inlineStr"/>
+      <c r="E16" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.dart.A3.png</t>
+        </is>
+      </c>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.dart.A3.json</t>
+        </is>
+      </c>
       <c r="G16" s="7" t="n">
-        <v>44</v>
+        <v>44.6</v>
       </c>
       <c r="H16" s="7" t="n">
-        <v>54</v>
+        <v>46.5</v>
       </c>
       <c r="I16" s="7" t="n">
         <v>0.5</v>
@@ -8007,13 +8015,21 @@
           <t>P3</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr"/>
-      <c r="F17" s="8" t="inlineStr"/>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.dart.A6.png</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.dart.A6.json</t>
+        </is>
+      </c>
       <c r="G17" s="7" t="n">
-        <v>48</v>
+        <v>62.8</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>58</v>
+        <v>67.2</v>
       </c>
       <c r="I17" s="7" t="n">
         <v>0.5</v>
@@ -10419,10 +10435,10 @@
         </is>
       </c>
       <c r="G66" s="7" t="n">
-        <v>13</v>
+        <v>19.1</v>
       </c>
       <c r="H66" s="7" t="n">
-        <v>13</v>
+        <v>19.1</v>
       </c>
       <c r="I66" s="7" t="n">
         <v>0.5</v>
@@ -10787,57 +10803,513 @@
         <v/>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>tower.dart.A1</t>
+        </is>
+      </c>
+      <c r="B74" s="9" t="inlineStr">
+        <is>
+          <t>装置变种</t>
+        </is>
+      </c>
+      <c r="C74" s="9" t="inlineStr">
+        <is>
+          <t>易拉罐投手「重罐点名」1 级挂件：挂一个秤砣</t>
+        </is>
+      </c>
+      <c r="D74" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E74" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.dart.A1.png</t>
+        </is>
+      </c>
+      <c r="F74" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.dart.A1.json</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="H74" s="7" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="I74" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J74" s="7" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="K74" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M74" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N74" s="9">
+        <f>IF(K74&gt;1,K74*G74*3&amp;" × "&amp;H74*3&amp;"（"&amp;K74&amp;" 帧横排）",G74*3&amp;" × "&amp;H74*3)</f>
+        <v/>
+      </c>
+    </row>
     <row r="75">
-      <c r="A75" s="10" t="inlineStr">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>tower.dart.A2</t>
+        </is>
+      </c>
+      <c r="B75" s="9" t="inlineStr">
+        <is>
+          <t>装置变种</t>
+        </is>
+      </c>
+      <c r="C75" s="9" t="inlineStr">
+        <is>
+          <t>易拉罐投手「重罐点名」2 级挂件：两侧各挂一个秤砣</t>
+        </is>
+      </c>
+      <c r="D75" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.dart.A2.png</t>
+        </is>
+      </c>
+      <c r="F75" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.dart.A2.json</t>
+        </is>
+      </c>
+      <c r="G75" s="7" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="H75" s="7" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="I75" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J75" s="7" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="K75" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L75" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N75" s="9">
+        <f>IF(K75&gt;1,K75*G75*3&amp;" × "&amp;H75*3&amp;"（"&amp;K75&amp;" 帧横排）",G75*3&amp;" × "&amp;H75*3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>shot.dart.A3</t>
+        </is>
+      </c>
+      <c r="B76" s="9" t="inlineStr">
+        <is>
+          <t>子弹</t>
+        </is>
+      </c>
+      <c r="C76" s="9" t="inlineStr">
+        <is>
+          <t>投掷物「重罐点名」3 级：蓄力铜罐</t>
+        </is>
+      </c>
+      <c r="D76" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E76" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.dart.A3.png</t>
+        </is>
+      </c>
+      <c r="F76" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.dart.A3.json</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="H76" s="7" t="n">
+        <v>21.2</v>
+      </c>
+      <c r="I76" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J76" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K76" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N76" s="9">
+        <f>IF(K76&gt;1,K76*G76*3&amp;" × "&amp;H76*3&amp;"（"&amp;K76&amp;" 帧横排）",G76*3&amp;" × "&amp;H76*3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>tower.dart.A4</t>
+        </is>
+      </c>
+      <c r="B77" s="9" t="inlineStr">
+        <is>
+          <t>装置变种</t>
+        </is>
+      </c>
+      <c r="C77" s="9" t="inlineStr">
+        <is>
+          <t>易拉罐投手「重罐点名」4 级：破防刺罐</t>
+        </is>
+      </c>
+      <c r="D77" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.dart.A4.png</t>
+        </is>
+      </c>
+      <c r="F77" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.dart.A4.json</t>
+        </is>
+      </c>
+      <c r="G77" s="7" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="H77" s="7" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="I77" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J77" s="7" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="K77" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L77" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N77" s="9">
+        <f>IF(K77&gt;1,K77*G77*3&amp;" × "&amp;H77*3&amp;"（"&amp;K77&amp;" 帧横排）",G77*3&amp;" × "&amp;H77*3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="inlineStr">
+        <is>
+          <t>shot.dart.A4</t>
+        </is>
+      </c>
+      <c r="B78" s="9" t="inlineStr">
+        <is>
+          <t>子弹</t>
+        </is>
+      </c>
+      <c r="C78" s="9" t="inlineStr">
+        <is>
+          <t>投掷物「重罐点名」4 级：破防刺罐</t>
+        </is>
+      </c>
+      <c r="D78" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E78" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.dart.A4.png</t>
+        </is>
+      </c>
+      <c r="F78" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.dart.A4.json</t>
+        </is>
+      </c>
+      <c r="G78" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="H78" s="7" t="n">
+        <v>21</v>
+      </c>
+      <c r="I78" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J78" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K78" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L78" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N78" s="9">
+        <f>IF(K78&gt;1,K78*G78*3&amp;" × "&amp;H78*3&amp;"（"&amp;K78&amp;" 帧横排）",G78*3&amp;" × "&amp;H78*3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>tower.dart.A5</t>
+        </is>
+      </c>
+      <c r="B79" s="9" t="inlineStr">
+        <is>
+          <t>装置变种</t>
+        </is>
+      </c>
+      <c r="C79" s="9" t="inlineStr">
+        <is>
+          <t>易拉罐投手「重罐点名」5 级：手雷</t>
+        </is>
+      </c>
+      <c r="D79" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.dart.A5.png</t>
+        </is>
+      </c>
+      <c r="F79" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.dart.A5.json</t>
+        </is>
+      </c>
+      <c r="G79" s="7" t="n">
+        <v>44.6</v>
+      </c>
+      <c r="H79" s="7" t="n">
+        <v>46.5</v>
+      </c>
+      <c r="I79" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J79" s="7" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="K79" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N79" s="9">
+        <f>IF(K79&gt;1,K79*G79*3&amp;" × "&amp;H79*3&amp;"（"&amp;K79&amp;" 帧横排）",G79*3&amp;" × "&amp;H79*3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="inlineStr">
+        <is>
+          <t>shot.dart.A5</t>
+        </is>
+      </c>
+      <c r="B80" s="9" t="inlineStr">
+        <is>
+          <t>子弹</t>
+        </is>
+      </c>
+      <c r="C80" s="9" t="inlineStr">
+        <is>
+          <t>投掷物「重罐点名」5 级：手雷</t>
+        </is>
+      </c>
+      <c r="D80" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E80" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.dart.A5.png</t>
+        </is>
+      </c>
+      <c r="F80" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.dart.A5.json</t>
+        </is>
+      </c>
+      <c r="G80" s="7" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="H80" s="7" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="I80" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J80" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K80" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L80" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N80" s="9">
+        <f>IF(K80&gt;1,K80*G80*3&amp;" × "&amp;H80*3&amp;"（"&amp;K80&amp;" 帧横排）",G80*3&amp;" × "&amp;H80*3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>shot.dart.A6</t>
+        </is>
+      </c>
+      <c r="B81" s="9" t="inlineStr">
+        <is>
+          <t>子弹</t>
+        </is>
+      </c>
+      <c r="C81" s="9" t="inlineStr">
+        <is>
+          <t>投掷物「重罐点名」6 级：双层底座 + 陨石</t>
+        </is>
+      </c>
+      <c r="D81" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.dart.A6.png</t>
+        </is>
+      </c>
+      <c r="F81" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.dart.A6.json</t>
+        </is>
+      </c>
+      <c r="G81" s="7" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="H81" s="7" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="I81" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J81" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K81" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L81" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N81" s="9">
+        <f>IF(K81&gt;1,K81*G81*3&amp;" × "&amp;H81*3&amp;"（"&amp;K81&amp;" 帧横排）",G81*3&amp;" × "&amp;H81*3)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="10" t="inlineStr">
         <is>
           <t>※ 图片地址填公开可访问的 https:// 链接（PNG / WebP，透明背景）；也可以不填，直接在游戏页面点「导入美术图片」，把文件名改成资源编号（如 tower.dart.png）一次选多张。</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="10" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="10" t="inlineStr">
         <is>
           <t>※ 游戏内宽高以 360 × 600 的画布为单位；出图按 3 倍像素（见最后一列），游戏会缩放到这里填的尺寸。</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="10" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="10" t="inlineStr">
         <is>
           <t>※ 锚点是图片里对齐游戏坐标的那一点：0,0 = 左上角，0.5,1 = 底边中点（跑者、装置用脚底中点）。</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="10" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="10" t="inlineStr">
         <is>
           <t>※ 帧数 &gt; 1 时，图片是横向排开的序列帧（每帧等宽），按帧率循环播放。跑者、Boss 统一画成「侧面向右跑」，向左时游戏自动水平翻转。</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="10" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="10" t="inlineStr">
         <is>
           <t>※ 装置变种图 tower.xxx.A3 / A6（B、C 同理）：该路线成为主路线并升到 3 级 / 6 级时替换基础图；没给就往下找，最后用基础图。导入时文件名里的装置也可以写 can / banana / sprinkler / drone / speaker / chill。</t>
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="10" t="inlineStr">
+    <row r="88">
+      <c r="A88" s="10" t="inlineStr">
         <is>
           <t>※ 动画：PNG 精灵图 + 同名 JSON（Aseprite「导出精灵图」勾选 JSON Data，或 TexturePacker JSON）。动画段用 Tag：idle 待机、fire 发射、build 放置、fly 子弹飞行、hit 命中；再用 1 帧的 release Tag 标出子弹离手的那一帧。用 Slice 标点：pivot 脚底 / 中心，muzzle 子弹出手点。导入时把 PNG 和 JSON 一起选上即可，或在「动画 JSON 地址」填链接。</t>
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" s="10" t="inlineStr">
+    <row r="89">
+      <c r="A89" s="10" t="inlineStr">
         <is>
           <t>※ 子弹只画外观：fly 画朝右，游戏沿弹道自动旋转；弹道类型、速度、抛物线高度在「弹道」表里调。</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="10" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="10" t="inlineStr">
         <is>
           <t>※ 优先级：P1 样板关（先画这些就能完整玩一张图）→ P2 → P3。</t>
         </is>
@@ -10845,7 +11317,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="M3:M73" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="M3:M81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"0,1"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Four towers' base looks from the concept sheets: banana tosser, dance speaker, sprinkler, shoebox drone (sheets, projectiles, drone flight); fix tesla shot counter overwriting the footprint size
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019aYuPSmDStWHRUCSamkHbW
</commit_message>
<xml_diff>
--- a/config/blast-track-config.xlsx
+++ b/config/blast-track-config.xlsx
@@ -7145,7 +7145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N90"/>
+  <dimension ref="A1:N91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7664,13 +7664,21 @@
           <t>P1 样板关</t>
         </is>
       </c>
-      <c r="E10" s="8" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr"/>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.bomb.png</t>
+        </is>
+      </c>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.bomb.json</t>
+        </is>
+      </c>
       <c r="G10" s="7" t="n">
-        <v>40</v>
+        <v>44.6</v>
       </c>
       <c r="H10" s="7" t="n">
-        <v>50</v>
+        <v>46.5</v>
       </c>
       <c r="I10" s="7" t="n">
         <v>0.5</v>
@@ -7713,13 +7721,21 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr"/>
-      <c r="F11" s="8" t="inlineStr"/>
+      <c r="E11" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.frost.png</t>
+        </is>
+      </c>
+      <c r="F11" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.frost.json</t>
+        </is>
+      </c>
       <c r="G11" s="7" t="n">
-        <v>40</v>
+        <v>78.2</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="I11" s="7" t="n">
         <v>0.5</v>
@@ -7762,13 +7778,21 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E12" s="8" t="inlineStr"/>
-      <c r="F12" s="8" t="inlineStr"/>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.sniper.png</t>
+        </is>
+      </c>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.sniper.json</t>
+        </is>
+      </c>
       <c r="G12" s="7" t="n">
-        <v>40</v>
+        <v>48.9</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>50</v>
+        <v>40.5</v>
       </c>
       <c r="I12" s="7" t="n">
         <v>0.5</v>
@@ -7811,13 +7835,21 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr"/>
-      <c r="F13" s="8" t="inlineStr"/>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.tesla.png</t>
+        </is>
+      </c>
+      <c r="F13" s="8" t="inlineStr">
+        <is>
+          <t>art/tower.tesla.json</t>
+        </is>
+      </c>
       <c r="G13" s="7" t="n">
-        <v>40</v>
+        <v>62.3</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>50</v>
+        <v>55.5</v>
       </c>
       <c r="I13" s="7" t="n">
         <v>0.5</v>
@@ -10481,13 +10513,21 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E67" s="8" t="inlineStr"/>
-      <c r="F67" s="8" t="inlineStr"/>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.bomb.png</t>
+        </is>
+      </c>
+      <c r="F67" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.bomb.json</t>
+        </is>
+      </c>
       <c r="G67" s="7" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H67" s="7" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I67" s="7" t="n">
         <v>0.5</v>
@@ -10530,13 +10570,21 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E68" s="8" t="inlineStr"/>
-      <c r="F68" s="8" t="inlineStr"/>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.sniper.png</t>
+        </is>
+      </c>
+      <c r="F68" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.sniper.json</t>
+        </is>
+      </c>
       <c r="G68" s="7" t="n">
-        <v>16</v>
+        <v>19.1</v>
       </c>
       <c r="H68" s="7" t="n">
-        <v>12</v>
+        <v>19.1</v>
       </c>
       <c r="I68" s="7" t="n">
         <v>0.5</v>
@@ -10579,7 +10627,11 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E69" s="8" t="inlineStr"/>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>art/fx.peel.png</t>
+        </is>
+      </c>
       <c r="F69" s="8" t="inlineStr"/>
       <c r="G69" s="7" t="n">
         <v>18</v>
@@ -11259,65 +11311,122 @@
         <v/>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="10" t="inlineStr">
-        <is>
-          <t>※ 图片地址填公开可访问的 https:// 链接（PNG / WebP，透明背景）；也可以不填，直接在游戏页面点「导入美术图片」，把文件名改成资源编号（如 tower.dart.png）一次选多张。</t>
-        </is>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
+          <t>fx.drone</t>
+        </is>
+      </c>
+      <c r="B82" s="9" t="inlineStr">
+        <is>
+          <t>特效</t>
+        </is>
+      </c>
+      <c r="C82" s="9" t="inlineStr">
+        <is>
+          <t>鞋盒无人机送货飞行（fly 循环，pivot 在机身中心）</t>
+        </is>
+      </c>
+      <c r="D82" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t>art/fx.drone.png</t>
+        </is>
+      </c>
+      <c r="F82" s="8" t="inlineStr">
+        <is>
+          <t>art/fx.drone.json</t>
+        </is>
+      </c>
+      <c r="G82" s="7" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="H82" s="7" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="I82" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J82" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K82" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L82" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N82" s="9">
+        <f>IF(K82&gt;1,K82*G82*3&amp;" × "&amp;H82*3&amp;"（"&amp;K82&amp;" 帧横排）",G82*3&amp;" × "&amp;H82*3)</f>
+        <v/>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
         <is>
-          <t>※ 游戏内宽高以 360 × 600 的画布为单位；出图按 3 倍像素（见最后一列），游戏会缩放到这里填的尺寸。</t>
+          <t>※ 图片地址填公开可访问的 https:// 链接（PNG / WebP，透明背景）；也可以不填，直接在游戏页面点「导入美术图片」，把文件名改成资源编号（如 tower.dart.png）一次选多张。</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>※ 锚点是图片里对齐游戏坐标的那一点：0,0 = 左上角，0.5,1 = 底边中点（跑者、装置用脚底中点）。</t>
+          <t>※ 游戏内宽高以 360 × 600 的画布为单位；出图按 3 倍像素（见最后一列），游戏会缩放到这里填的尺寸。</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>※ 帧数 &gt; 1 时，图片是横向排开的序列帧（每帧等宽），按帧率循环播放。跑者、Boss 统一画成「侧面向右跑」，向左时游戏自动水平翻转。</t>
+          <t>※ 锚点是图片里对齐游戏坐标的那一点：0,0 = 左上角，0.5,1 = 底边中点（跑者、装置用脚底中点）。</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>※ 装置变种图 tower.xxx.A3 / A6（B、C 同理）：该路线成为主路线并升到 3 级 / 6 级时替换基础图；没给就往下找，最后用基础图。导入时文件名里的装置也可以写 can / banana / sprinkler / drone / speaker / chill。</t>
+          <t>※ 帧数 &gt; 1 时，图片是横向排开的序列帧（每帧等宽），按帧率循环播放。跑者、Boss 统一画成「侧面向右跑」，向左时游戏自动水平翻转。</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>※ 动画：PNG 精灵图 + 同名 JSON（Aseprite「导出精灵图」勾选 JSON Data，或 TexturePacker JSON）。动画段用 Tag：idle 待机、fire 发射、build 放置、fly 子弹飞行、hit 命中；再用 1 帧的 release Tag 标出子弹离手的那一帧。用 Slice 标点：pivot 脚底 / 中心，muzzle 子弹出手点。导入时把 PNG 和 JSON 一起选上即可，或在「动画 JSON 地址」填链接。</t>
+          <t>※ 装置变种图 tower.xxx.A3 / A6（B、C 同理）：该路线成为主路线并升到 3 级 / 6 级时替换基础图；没给就往下找，最后用基础图。导入时文件名里的装置也可以写 can / banana / sprinkler / drone / speaker / chill。</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>※ 子弹只画外观：fly 画朝右，游戏沿弹道自动旋转；弹道类型、速度、抛物线高度在「弹道」表里调。</t>
+          <t>※ 动画：PNG 精灵图 + 同名 JSON（Aseprite「导出精灵图」勾选 JSON Data，或 TexturePacker JSON）。动画段用 Tag：idle 待机、fire 发射、build 放置、fly 子弹飞行、hit 命中；再用 1 帧的 release Tag 标出子弹离手的那一帧。用 Slice 标点：pivot 脚底 / 中心，muzzle 子弹出手点。导入时把 PNG 和 JSON 一起选上即可，或在「动画 JSON 地址」填链接。</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
         <is>
+          <t>※ 子弹只画外观：fly 画朝右，游戏沿弹道自动旋转；弹道类型、速度、抛物线高度在「弹道」表里调。</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="10" t="inlineStr">
+        <is>
           <t>※ 优先级：P1 样板关（先画这些就能完整玩一张图）→ P2 → P3。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="M3:M81" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="M3:M82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"0,1"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Sprinkler head now spins and flings droplets; dance speaker sends out a spreading sound wave to its range
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019aYuPSmDStWHRUCSamkHbW
</commit_message>
<xml_diff>
--- a/config/blast-track-config.xlsx
+++ b/config/blast-track-config.xlsx
@@ -7732,10 +7732,10 @@
         </is>
       </c>
       <c r="G11" s="7" t="n">
-        <v>78.2</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="H11" s="7" t="n">
-        <v>43</v>
+        <v>50.5</v>
       </c>
       <c r="I11" s="7" t="n">
         <v>0.5</v>

</xml_diff>

<commit_message>
v21: sprinkler truck drives around its water station and sprays from where it is
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MSxiXd6jSsJas8jyd5R32w
</commit_message>
<xml_diff>
--- a/config/blast-track-config.xlsx
+++ b/config/blast-track-config.xlsx
@@ -1339,32 +1339,32 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>洒水器</t>
+          <t>洒水车</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>Sprinkler</t>
+          <t>Truck</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t>Arroseur</t>
+          <t>Camion</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>解锁洒水器：持续喷水，范围减速</t>
+          <t>解锁洒水车：持续喷水，范围减速</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>Unlock the Sprinkler: keeps spraying, slows an area</t>
+          <t>Unlock the Sprinkler Truck: drives around spraying, slows an area</t>
         </is>
       </c>
       <c r="K4" s="8" t="inlineStr">
         <is>
-          <t>Débloque l’Arroseur : arrose en continu et ralentit une zone</t>
+          <t>Débloque le Camion arroseur : il roule en arrosant et ralentit une zone</t>
         </is>
       </c>
       <c r="L4" s="7" t="n">
@@ -7145,7 +7145,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N91"/>
+  <dimension ref="A1:N92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -7713,7 +7713,7 @@
       </c>
       <c r="C11" s="9" t="inlineStr">
         <is>
-          <t>洒水器：基础造型，面朝右（朝左时游戏自动翻转）。可做动画：idle 待机 + fire 发射（JSON 标出 release 出手帧和 muzzle 出手点）</t>
+          <t>洒水车取水站：基础造型，面朝右（朝左时游戏自动翻转）。可做动画：idle 待机 + fire 发射（JSON 标出 release 出手帧和 muzzle 出手点）</t>
         </is>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -8586,7 +8586,7 @@
       </c>
       <c r="C28" s="9" t="inlineStr">
         <is>
-          <t>洒水器「喷淋湿地」主路线 3 级起的造型（A3；没有 A4、A5 时沿用 A3）</t>
+          <t>洒水车取水站「喷淋湿地」主路线 3 级起的造型（A3；没有 A4、A5 时沿用 A3）</t>
         </is>
       </c>
       <c r="D28" s="9" t="inlineStr">
@@ -8635,7 +8635,7 @@
       </c>
       <c r="C29" s="9" t="inlineStr">
         <is>
-          <t>洒水器「喷淋湿地」主路线 6 级起的造型（A6；没有 A4、A5 时沿用 A3）</t>
+          <t>洒水车取水站「喷淋湿地」主路线 6 级起的造型（A6；没有 A4、A5 时沿用 A3）</t>
         </is>
       </c>
       <c r="D29" s="9" t="inlineStr">
@@ -8684,7 +8684,7 @@
       </c>
       <c r="C30" s="9" t="inlineStr">
         <is>
-          <t>洒水器「寒霜喷头」主路线 3 级起的造型（B3；没有 B4、B5 时沿用 B3）</t>
+          <t>洒水车取水站「寒霜喷头」主路线 3 级起的造型（B3；没有 B4、B5 时沿用 B3）</t>
         </is>
       </c>
       <c r="D30" s="9" t="inlineStr">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="C31" s="9" t="inlineStr">
         <is>
-          <t>洒水器「寒霜喷头」主路线 6 级起的造型（B6；没有 B4、B5 时沿用 B3）</t>
+          <t>洒水车取水站「寒霜喷头」主路线 6 级起的造型（B6；没有 B4、B5 时沿用 B3）</t>
         </is>
       </c>
       <c r="D31" s="9" t="inlineStr">
@@ -8782,7 +8782,7 @@
       </c>
       <c r="C32" s="9" t="inlineStr">
         <is>
-          <t>洒水器「高压水柱」主路线 3 级起的造型（C3；没有 C4、C5 时沿用 C3）</t>
+          <t>洒水车取水站「高压水柱」主路线 3 级起的造型（C3；没有 C4、C5 时沿用 C3）</t>
         </is>
       </c>
       <c r="D32" s="9" t="inlineStr">
@@ -8831,7 +8831,7 @@
       </c>
       <c r="C33" s="9" t="inlineStr">
         <is>
-          <t>洒水器「高压水柱」主路线 6 级起的造型（C6；没有 C4、C5 时沿用 C3）</t>
+          <t>洒水车取水站「高压水柱」主路线 6 级起的造型（C6；没有 C4、C5 时沿用 C3）</t>
         </is>
       </c>
       <c r="D33" s="9" t="inlineStr">
@@ -9752,37 +9752,41 @@
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>pad.empty</t>
+          <t>truck.frost</t>
         </is>
       </c>
       <c r="B52" s="9" t="inlineStr">
         <is>
-          <t>空位</t>
+          <t>装置</t>
         </is>
       </c>
       <c r="C52" s="9" t="inlineStr">
         <is>
-          <t>可放置装置的空位（石台 + 加号）</t>
+          <t>洒水车：会开的车，车头朝右（朝左时游戏自动翻转），地面点在车轮下；静态图即可，行驶时游戏会让它颠簸，喷水从车头喷口出；tower.frost（洒水器）画在它的停车位上当取水站</t>
         </is>
       </c>
       <c r="D52" s="9" t="inlineStr">
         <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="E52" s="8" t="inlineStr"/>
+          <t>P1 样板关</t>
+        </is>
+      </c>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t>art/truck.frost.png</t>
+        </is>
+      </c>
       <c r="F52" s="8" t="inlineStr"/>
       <c r="G52" s="7" t="n">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="H52" s="7" t="n">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="I52" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="J52" s="7" t="n">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="K52" s="7" t="n">
         <v>1</v>
@@ -9801,7 +9805,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>pad.base</t>
+          <t>pad.empty</t>
         </is>
       </c>
       <c r="B53" s="9" t="inlineStr">
@@ -9811,7 +9815,7 @@
       </c>
       <c r="C53" s="9" t="inlineStr">
         <is>
-          <t>装置脚下的底座</t>
+          <t>可放置装置的空位（石台 + 加号）</t>
         </is>
       </c>
       <c r="D53" s="9" t="inlineStr">
@@ -9850,31 +9854,31 @@
     <row r="54">
       <c r="A54" s="6" t="inlineStr">
         <is>
-          <t>runner.norm</t>
+          <t>pad.base</t>
         </is>
       </c>
       <c r="B54" s="9" t="inlineStr">
         <is>
-          <t>跑者</t>
+          <t>空位</t>
         </is>
       </c>
       <c r="C54" s="9" t="inlineStr">
         <is>
-          <t>慢跑者，侧面向右跑；横向序列帧</t>
+          <t>装置脚下的底座</t>
         </is>
       </c>
       <c r="D54" s="9" t="inlineStr">
         <is>
-          <t>P1 样板关</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr"/>
       <c r="F54" s="8" t="inlineStr"/>
       <c r="G54" s="7" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="H54" s="7" t="n">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="I54" s="7" t="n">
         <v>0.5</v>
@@ -9883,10 +9887,10 @@
         <v>1</v>
       </c>
       <c r="K54" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="L54" s="7" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="M54" s="7" t="n">
         <v>0</v>
@@ -9899,7 +9903,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>runner.arm</t>
+          <t>runner.norm</t>
         </is>
       </c>
       <c r="B55" s="9" t="inlineStr">
@@ -9909,7 +9913,7 @@
       </c>
       <c r="C55" s="9" t="inlineStr">
         <is>
-          <t>耐力跑者（更壮、带护具）</t>
+          <t>慢跑者，侧面向右跑；横向序列帧</t>
         </is>
       </c>
       <c r="D55" s="9" t="inlineStr">
@@ -9920,10 +9924,10 @@
       <c r="E55" s="8" t="inlineStr"/>
       <c r="F55" s="8" t="inlineStr"/>
       <c r="G55" s="7" t="n">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="H55" s="7" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="I55" s="7" t="n">
         <v>0.5</v>
@@ -9948,7 +9952,7 @@
     <row r="56">
       <c r="A56" s="6" t="inlineStr">
         <is>
-          <t>runner.mini</t>
+          <t>runner.arm</t>
         </is>
       </c>
       <c r="B56" s="9" t="inlineStr">
@@ -9958,21 +9962,21 @@
       </c>
       <c r="C56" s="9" t="inlineStr">
         <is>
-          <t>跑团分裂出的小跑者</t>
+          <t>耐力跑者（更壮、带护具）</t>
         </is>
       </c>
       <c r="D56" s="9" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1 样板关</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr"/>
       <c r="F56" s="8" t="inlineStr"/>
       <c r="G56" s="7" t="n">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="H56" s="7" t="n">
-        <v>26</v>
+        <v>42</v>
       </c>
       <c r="I56" s="7" t="n">
         <v>0.5</v>
@@ -9984,7 +9988,7 @@
         <v>6</v>
       </c>
       <c r="L56" s="7" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="M56" s="7" t="n">
         <v>0</v>
@@ -9997,7 +10001,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>runner.gold</t>
+          <t>runner.mini</t>
         </is>
       </c>
       <c r="B57" s="9" t="inlineStr">
@@ -10007,7 +10011,7 @@
       </c>
       <c r="C57" s="9" t="inlineStr">
         <is>
-          <t>Aurum 召唤的金甲跑者</t>
+          <t>跑团分裂出的小跑者</t>
         </is>
       </c>
       <c r="D57" s="9" t="inlineStr">
@@ -10018,10 +10022,10 @@
       <c r="E57" s="8" t="inlineStr"/>
       <c r="F57" s="8" t="inlineStr"/>
       <c r="G57" s="7" t="n">
-        <v>32</v>
+        <v>22</v>
       </c>
       <c r="H57" s="7" t="n">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="I57" s="7" t="n">
         <v>0.5</v>
@@ -10033,7 +10037,7 @@
         <v>6</v>
       </c>
       <c r="L57" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="M57" s="7" t="n">
         <v>0</v>
@@ -10046,31 +10050,31 @@
     <row r="58">
       <c r="A58" s="6" t="inlineStr">
         <is>
-          <t>boss.yawn</t>
+          <t>runner.gold</t>
         </is>
       </c>
       <c r="B58" s="9" t="inlineStr">
         <is>
-          <t>Boss</t>
+          <t>跑者</t>
         </is>
       </c>
       <c r="C58" s="9" t="inlineStr">
         <is>
-          <t>Nox（黑猫，九命），侧面向右跑；真人原型需本人同意</t>
+          <t>Aurum 召唤的金甲跑者</t>
         </is>
       </c>
       <c r="D58" s="9" t="inlineStr">
         <is>
-          <t>P1 样板关</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr"/>
       <c r="F58" s="8" t="inlineStr"/>
       <c r="G58" s="7" t="n">
-        <v>72</v>
+        <v>32</v>
       </c>
       <c r="H58" s="7" t="n">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="I58" s="7" t="n">
         <v>0.5</v>
@@ -10082,7 +10086,7 @@
         <v>6</v>
       </c>
       <c r="L58" s="7" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M58" s="7" t="n">
         <v>0</v>
@@ -10095,7 +10099,7 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>boss.gilg</t>
+          <t>boss.yawn</t>
         </is>
       </c>
       <c r="B59" s="9" t="inlineStr">
@@ -10105,21 +10109,21 @@
       </c>
       <c r="C59" s="9" t="inlineStr">
         <is>
-          <t>Aurum，侧面向右跑；真人原型需本人同意</t>
+          <t>Nox（黑猫，九命），侧面向右跑；真人原型需本人同意</t>
         </is>
       </c>
       <c r="D59" s="9" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>P1 样板关</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr"/>
       <c r="F59" s="8" t="inlineStr"/>
       <c r="G59" s="7" t="n">
-        <v>64</v>
+        <v>72</v>
       </c>
       <c r="H59" s="7" t="n">
-        <v>80</v>
+        <v>56</v>
       </c>
       <c r="I59" s="7" t="n">
         <v>0.5</v>
@@ -10144,7 +10148,7 @@
     <row r="60">
       <c r="A60" s="6" t="inlineStr">
         <is>
-          <t>boss.king</t>
+          <t>boss.gilg</t>
         </is>
       </c>
       <c r="B60" s="9" t="inlineStr">
@@ -10154,7 +10158,7 @@
       </c>
       <c r="C60" s="9" t="inlineStr">
         <is>
-          <t>Slimo，侧面向右跑；真人原型需本人同意</t>
+          <t>Aurum，侧面向右跑；真人原型需本人同意</t>
         </is>
       </c>
       <c r="D60" s="9" t="inlineStr">
@@ -10193,7 +10197,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>boss.lucas</t>
+          <t>boss.king</t>
         </is>
       </c>
       <c r="B61" s="9" t="inlineStr">
@@ -10203,7 +10207,7 @@
       </c>
       <c r="C61" s="9" t="inlineStr">
         <is>
-          <t>Rocco，侧面向右跑；真人原型需本人同意</t>
+          <t>Slimo，侧面向右跑；真人原型需本人同意</t>
         </is>
       </c>
       <c r="D61" s="9" t="inlineStr">
@@ -10242,7 +10246,7 @@
     <row r="62">
       <c r="A62" s="6" t="inlineStr">
         <is>
-          <t>boss.shiti</t>
+          <t>boss.lucas</t>
         </is>
       </c>
       <c r="B62" s="9" t="inlineStr">
@@ -10252,7 +10256,7 @@
       </c>
       <c r="C62" s="9" t="inlineStr">
         <is>
-          <t>Chuckles，侧面向右跑；真人原型需本人同意</t>
+          <t>Rocco，侧面向右跑；真人原型需本人同意</t>
         </is>
       </c>
       <c r="D62" s="9" t="inlineStr">
@@ -10291,7 +10295,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>boss.jerry</t>
+          <t>boss.shiti</t>
         </is>
       </c>
       <c r="B63" s="9" t="inlineStr">
@@ -10301,7 +10305,7 @@
       </c>
       <c r="C63" s="9" t="inlineStr">
         <is>
-          <t>Datto，侧面向右跑；真人原型需本人同意</t>
+          <t>Chuckles，侧面向右跑；真人原型需本人同意</t>
         </is>
       </c>
       <c r="D63" s="9" t="inlineStr">
@@ -10340,7 +10344,7 @@
     <row r="64">
       <c r="A64" s="6" t="inlineStr">
         <is>
-          <t>boss.pizza</t>
+          <t>boss.jerry</t>
         </is>
       </c>
       <c r="B64" s="9" t="inlineStr">
@@ -10350,7 +10354,7 @@
       </c>
       <c r="C64" s="9" t="inlineStr">
         <is>
-          <t>Pizza Rider（披萨外卖员），侧面向右跑；真人原型需本人同意</t>
+          <t>Datto，侧面向右跑；真人原型需本人同意</t>
         </is>
       </c>
       <c r="D64" s="9" t="inlineStr">
@@ -10389,7 +10393,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>boss.overflow</t>
+          <t>boss.pizza</t>
         </is>
       </c>
       <c r="B65" s="9" t="inlineStr">
@@ -10399,7 +10403,7 @@
       </c>
       <c r="C65" s="9" t="inlineStr">
         <is>
-          <t>Overflow（溢出怪），侧面向右跑；真人原型需本人同意</t>
+          <t>Pizza Rider（披萨外卖员），侧面向右跑；真人原型需本人同意</t>
         </is>
       </c>
       <c r="D65" s="9" t="inlineStr">
@@ -10438,17 +10442,17 @@
     <row r="66">
       <c r="A66" s="6" t="inlineStr">
         <is>
-          <t>shot.dart</t>
+          <t>boss.overflow</t>
         </is>
       </c>
       <c r="B66" s="9" t="inlineStr">
         <is>
-          <t>子弹</t>
+          <t>Boss</t>
         </is>
       </c>
       <c r="C66" s="9" t="inlineStr">
         <is>
-          <t>易拉罐：fly 飞行循环（画朝右，游戏沿弹道旋转）+ hit 命中</t>
+          <t>Overflow（溢出怪），侧面向右跑；真人原型需本人同意</t>
         </is>
       </c>
       <c r="D66" s="9" t="inlineStr">
@@ -10456,33 +10460,25 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E66" s="8" t="inlineStr">
-        <is>
-          <t>art/shot.dart.png</t>
-        </is>
-      </c>
-      <c r="F66" s="8" t="inlineStr">
-        <is>
-          <t>art/shot.dart.json</t>
-        </is>
-      </c>
+      <c r="E66" s="8" t="inlineStr"/>
+      <c r="F66" s="8" t="inlineStr"/>
       <c r="G66" s="7" t="n">
-        <v>19.1</v>
+        <v>64</v>
       </c>
       <c r="H66" s="7" t="n">
-        <v>19.1</v>
+        <v>80</v>
       </c>
       <c r="I66" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="J66" s="7" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K66" s="7" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L66" s="7" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="M66" s="7" t="n">
         <v>0</v>
@@ -10495,7 +10491,7 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>shot.bomb</t>
+          <t>shot.dart</t>
         </is>
       </c>
       <c r="B67" s="9" t="inlineStr">
@@ -10505,7 +10501,7 @@
       </c>
       <c r="C67" s="9" t="inlineStr">
         <is>
-          <t>飞行中的香蕉皮：fly + hit（落地）</t>
+          <t>易拉罐：fly 飞行循环（画朝右，游戏沿弹道旋转）+ hit 命中</t>
         </is>
       </c>
       <c r="D67" s="9" t="inlineStr">
@@ -10515,19 +10511,19 @@
       </c>
       <c r="E67" s="8" t="inlineStr">
         <is>
-          <t>art/shot.bomb.png</t>
+          <t>art/shot.dart.png</t>
         </is>
       </c>
       <c r="F67" s="8" t="inlineStr">
         <is>
-          <t>art/shot.bomb.json</t>
+          <t>art/shot.dart.json</t>
         </is>
       </c>
       <c r="G67" s="7" t="n">
-        <v>15</v>
+        <v>19.1</v>
       </c>
       <c r="H67" s="7" t="n">
-        <v>15</v>
+        <v>19.1</v>
       </c>
       <c r="I67" s="7" t="n">
         <v>0.5</v>
@@ -10552,7 +10548,7 @@
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>shot.sniper</t>
+          <t>shot.bomb</t>
         </is>
       </c>
       <c r="B68" s="9" t="inlineStr">
@@ -10562,7 +10558,7 @@
       </c>
       <c r="C68" s="9" t="inlineStr">
         <is>
-          <t>无人机空投的鞋盒：fly（下落）+ hit（砸地）</t>
+          <t>飞行中的香蕉皮：fly + hit（落地）</t>
         </is>
       </c>
       <c r="D68" s="9" t="inlineStr">
@@ -10572,25 +10568,25 @@
       </c>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t>art/shot.sniper.png</t>
+          <t>art/shot.bomb.png</t>
         </is>
       </c>
       <c r="F68" s="8" t="inlineStr">
         <is>
-          <t>art/shot.sniper.json</t>
+          <t>art/shot.bomb.json</t>
         </is>
       </c>
       <c r="G68" s="7" t="n">
-        <v>19.1</v>
+        <v>15</v>
       </c>
       <c r="H68" s="7" t="n">
-        <v>19.1</v>
+        <v>15</v>
       </c>
       <c r="I68" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="J68" s="7" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="K68" s="7" t="n">
         <v>1</v>
@@ -10609,17 +10605,17 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>fx.peel</t>
+          <t>shot.sniper</t>
         </is>
       </c>
       <c r="B69" s="9" t="inlineStr">
         <is>
-          <t>地面效果</t>
+          <t>子弹</t>
         </is>
       </c>
       <c r="C69" s="9" t="inlineStr">
         <is>
-          <t>落在跑道上的香蕉皮</t>
+          <t>无人机空投的鞋盒：fly（下落）+ hit（砸地）</t>
         </is>
       </c>
       <c r="D69" s="9" t="inlineStr">
@@ -10629,21 +10625,25 @@
       </c>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t>art/fx.peel.png</t>
-        </is>
-      </c>
-      <c r="F69" s="8" t="inlineStr"/>
+          <t>art/shot.sniper.png</t>
+        </is>
+      </c>
+      <c r="F69" s="8" t="inlineStr">
+        <is>
+          <t>art/shot.sniper.json</t>
+        </is>
+      </c>
       <c r="G69" s="7" t="n">
-        <v>18</v>
+        <v>19.1</v>
       </c>
       <c r="H69" s="7" t="n">
-        <v>18</v>
+        <v>19.1</v>
       </c>
       <c r="I69" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="J69" s="7" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="K69" s="7" t="n">
         <v>1</v>
@@ -10662,17 +10662,17 @@
     <row r="70">
       <c r="A70" s="6" t="inlineStr">
         <is>
-          <t>icon.wave</t>
+          <t>fx.peel</t>
         </is>
       </c>
       <c r="B70" s="9" t="inlineStr">
         <is>
-          <t>界面图标</t>
+          <t>地面效果</t>
         </is>
       </c>
       <c r="C70" s="9" t="inlineStr">
         <is>
-          <t>顶栏「波次」图标</t>
+          <t>落在跑道上的香蕉皮</t>
         </is>
       </c>
       <c r="D70" s="9" t="inlineStr">
@@ -10680,13 +10680,17 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E70" s="8" t="inlineStr"/>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t>art/fx.peel.png</t>
+        </is>
+      </c>
       <c r="F70" s="8" t="inlineStr"/>
       <c r="G70" s="7" t="n">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="H70" s="7" t="n">
-        <v>38</v>
+        <v>18</v>
       </c>
       <c r="I70" s="7" t="n">
         <v>0.5</v>
@@ -10711,7 +10715,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>icon.lives</t>
+          <t>icon.wave</t>
         </is>
       </c>
       <c r="B71" s="9" t="inlineStr">
@@ -10721,7 +10725,7 @@
       </c>
       <c r="C71" s="9" t="inlineStr">
         <is>
-          <t>顶栏「生命」图标（心形）</t>
+          <t>顶栏「波次」图标</t>
         </is>
       </c>
       <c r="D71" s="9" t="inlineStr">
@@ -10760,7 +10764,7 @@
     <row r="72">
       <c r="A72" s="6" t="inlineStr">
         <is>
-          <t>icon.gst</t>
+          <t>icon.lives</t>
         </is>
       </c>
       <c r="B72" s="9" t="inlineStr">
@@ -10770,7 +10774,7 @@
       </c>
       <c r="C72" s="9" t="inlineStr">
         <is>
-          <t>顶栏「GST」图标</t>
+          <t>顶栏「生命」图标（心形）</t>
         </is>
       </c>
       <c r="D72" s="9" t="inlineStr">
@@ -10809,7 +10813,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>icon.score</t>
+          <t>icon.gst</t>
         </is>
       </c>
       <c r="B73" s="9" t="inlineStr">
@@ -10819,7 +10823,7 @@
       </c>
       <c r="C73" s="9" t="inlineStr">
         <is>
-          <t>顶栏「分数」图标</t>
+          <t>顶栏「GST」图标</t>
         </is>
       </c>
       <c r="D73" s="9" t="inlineStr">
@@ -10858,17 +10862,17 @@
     <row r="74">
       <c r="A74" s="6" t="inlineStr">
         <is>
-          <t>tower.dart.A1</t>
+          <t>icon.score</t>
         </is>
       </c>
       <c r="B74" s="9" t="inlineStr">
         <is>
-          <t>装置变种</t>
+          <t>界面图标</t>
         </is>
       </c>
       <c r="C74" s="9" t="inlineStr">
         <is>
-          <t>易拉罐投手「重罐点名」1 级挂件：挂一个秤砣</t>
+          <t>顶栏「分数」图标</t>
         </is>
       </c>
       <c r="D74" s="9" t="inlineStr">
@@ -10876,27 +10880,19 @@
           <t>P2</t>
         </is>
       </c>
-      <c r="E74" s="8" t="inlineStr">
-        <is>
-          <t>art/tower.dart.A1.png</t>
-        </is>
-      </c>
-      <c r="F74" s="8" t="inlineStr">
-        <is>
-          <t>art/tower.dart.A1.json</t>
-        </is>
-      </c>
+      <c r="E74" s="8" t="inlineStr"/>
+      <c r="F74" s="8" t="inlineStr"/>
       <c r="G74" s="7" t="n">
-        <v>44.6</v>
+        <v>38</v>
       </c>
       <c r="H74" s="7" t="n">
-        <v>46.5</v>
+        <v>38</v>
       </c>
       <c r="I74" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="J74" s="7" t="n">
-        <v>0.92</v>
+        <v>0.5</v>
       </c>
       <c r="K74" s="7" t="n">
         <v>1</v>
@@ -10915,7 +10911,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>tower.dart.A2</t>
+          <t>tower.dart.A1</t>
         </is>
       </c>
       <c r="B75" s="9" t="inlineStr">
@@ -10925,7 +10921,7 @@
       </c>
       <c r="C75" s="9" t="inlineStr">
         <is>
-          <t>易拉罐投手「重罐点名」2 级挂件：两侧各挂一个秤砣</t>
+          <t>易拉罐投手「重罐点名」1 级挂件：挂一个秤砣</t>
         </is>
       </c>
       <c r="D75" s="9" t="inlineStr">
@@ -10935,12 +10931,12 @@
       </c>
       <c r="E75" s="8" t="inlineStr">
         <is>
-          <t>art/tower.dart.A2.png</t>
+          <t>art/tower.dart.A1.png</t>
         </is>
       </c>
       <c r="F75" s="8" t="inlineStr">
         <is>
-          <t>art/tower.dart.A2.json</t>
+          <t>art/tower.dart.A1.json</t>
         </is>
       </c>
       <c r="G75" s="7" t="n">
@@ -10972,17 +10968,17 @@
     <row r="76">
       <c r="A76" s="6" t="inlineStr">
         <is>
-          <t>shot.dart.A3</t>
+          <t>tower.dart.A2</t>
         </is>
       </c>
       <c r="B76" s="9" t="inlineStr">
         <is>
-          <t>子弹</t>
+          <t>装置变种</t>
         </is>
       </c>
       <c r="C76" s="9" t="inlineStr">
         <is>
-          <t>投掷物「重罐点名」3 级：蓄力铜罐</t>
+          <t>易拉罐投手「重罐点名」2 级挂件：两侧各挂一个秤砣</t>
         </is>
       </c>
       <c r="D76" s="9" t="inlineStr">
@@ -10992,25 +10988,25 @@
       </c>
       <c r="E76" s="8" t="inlineStr">
         <is>
-          <t>art/shot.dart.A3.png</t>
+          <t>art/tower.dart.A2.png</t>
         </is>
       </c>
       <c r="F76" s="8" t="inlineStr">
         <is>
-          <t>art/shot.dart.A3.json</t>
+          <t>art/tower.dart.A2.json</t>
         </is>
       </c>
       <c r="G76" s="7" t="n">
-        <v>21.2</v>
+        <v>44.6</v>
       </c>
       <c r="H76" s="7" t="n">
-        <v>21.2</v>
+        <v>46.5</v>
       </c>
       <c r="I76" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="J76" s="7" t="n">
-        <v>0.5</v>
+        <v>0.92</v>
       </c>
       <c r="K76" s="7" t="n">
         <v>1</v>
@@ -11029,17 +11025,17 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>tower.dart.A4</t>
+          <t>shot.dart.A3</t>
         </is>
       </c>
       <c r="B77" s="9" t="inlineStr">
         <is>
-          <t>装置变种</t>
+          <t>子弹</t>
         </is>
       </c>
       <c r="C77" s="9" t="inlineStr">
         <is>
-          <t>易拉罐投手「重罐点名」4 级：破防刺罐</t>
+          <t>投掷物「重罐点名」3 级：蓄力铜罐</t>
         </is>
       </c>
       <c r="D77" s="9" t="inlineStr">
@@ -11049,25 +11045,25 @@
       </c>
       <c r="E77" s="8" t="inlineStr">
         <is>
-          <t>art/tower.dart.A4.png</t>
+          <t>art/shot.dart.A3.png</t>
         </is>
       </c>
       <c r="F77" s="8" t="inlineStr">
         <is>
-          <t>art/tower.dart.A4.json</t>
+          <t>art/shot.dart.A3.json</t>
         </is>
       </c>
       <c r="G77" s="7" t="n">
-        <v>44.6</v>
+        <v>21.2</v>
       </c>
       <c r="H77" s="7" t="n">
-        <v>46.5</v>
+        <v>21.2</v>
       </c>
       <c r="I77" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="J77" s="7" t="n">
-        <v>0.92</v>
+        <v>0.5</v>
       </c>
       <c r="K77" s="7" t="n">
         <v>1</v>
@@ -11086,17 +11082,17 @@
     <row r="78">
       <c r="A78" s="6" t="inlineStr">
         <is>
-          <t>shot.dart.A4</t>
+          <t>tower.dart.A4</t>
         </is>
       </c>
       <c r="B78" s="9" t="inlineStr">
         <is>
-          <t>子弹</t>
+          <t>装置变种</t>
         </is>
       </c>
       <c r="C78" s="9" t="inlineStr">
         <is>
-          <t>投掷物「重罐点名」4 级：破防刺罐</t>
+          <t>易拉罐投手「重罐点名」4 级：破防刺罐</t>
         </is>
       </c>
       <c r="D78" s="9" t="inlineStr">
@@ -11106,25 +11102,25 @@
       </c>
       <c r="E78" s="8" t="inlineStr">
         <is>
-          <t>art/shot.dart.A4.png</t>
+          <t>art/tower.dart.A4.png</t>
         </is>
       </c>
       <c r="F78" s="8" t="inlineStr">
         <is>
-          <t>art/shot.dart.A4.json</t>
+          <t>art/tower.dart.A4.json</t>
         </is>
       </c>
       <c r="G78" s="7" t="n">
-        <v>21</v>
+        <v>44.6</v>
       </c>
       <c r="H78" s="7" t="n">
-        <v>21</v>
+        <v>46.5</v>
       </c>
       <c r="I78" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="J78" s="7" t="n">
-        <v>0.5</v>
+        <v>0.92</v>
       </c>
       <c r="K78" s="7" t="n">
         <v>1</v>
@@ -11143,17 +11139,17 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>tower.dart.A5</t>
+          <t>shot.dart.A4</t>
         </is>
       </c>
       <c r="B79" s="9" t="inlineStr">
         <is>
-          <t>装置变种</t>
+          <t>子弹</t>
         </is>
       </c>
       <c r="C79" s="9" t="inlineStr">
         <is>
-          <t>易拉罐投手「重罐点名」5 级：手雷</t>
+          <t>投掷物「重罐点名」4 级：破防刺罐</t>
         </is>
       </c>
       <c r="D79" s="9" t="inlineStr">
@@ -11163,25 +11159,25 @@
       </c>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t>art/tower.dart.A5.png</t>
+          <t>art/shot.dart.A4.png</t>
         </is>
       </c>
       <c r="F79" s="8" t="inlineStr">
         <is>
-          <t>art/tower.dart.A5.json</t>
+          <t>art/shot.dart.A4.json</t>
         </is>
       </c>
       <c r="G79" s="7" t="n">
-        <v>44.6</v>
+        <v>21</v>
       </c>
       <c r="H79" s="7" t="n">
-        <v>46.5</v>
+        <v>21</v>
       </c>
       <c r="I79" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="J79" s="7" t="n">
-        <v>0.92</v>
+        <v>0.5</v>
       </c>
       <c r="K79" s="7" t="n">
         <v>1</v>
@@ -11200,17 +11196,17 @@
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>shot.dart.A5</t>
+          <t>tower.dart.A5</t>
         </is>
       </c>
       <c r="B80" s="9" t="inlineStr">
         <is>
-          <t>子弹</t>
+          <t>装置变种</t>
         </is>
       </c>
       <c r="C80" s="9" t="inlineStr">
         <is>
-          <t>投掷物「重罐点名」5 级：手雷</t>
+          <t>易拉罐投手「重罐点名」5 级：手雷</t>
         </is>
       </c>
       <c r="D80" s="9" t="inlineStr">
@@ -11220,25 +11216,25 @@
       </c>
       <c r="E80" s="8" t="inlineStr">
         <is>
-          <t>art/shot.dart.A5.png</t>
+          <t>art/tower.dart.A5.png</t>
         </is>
       </c>
       <c r="F80" s="8" t="inlineStr">
         <is>
-          <t>art/shot.dart.A5.json</t>
+          <t>art/tower.dart.A5.json</t>
         </is>
       </c>
       <c r="G80" s="7" t="n">
-        <v>23.4</v>
+        <v>44.6</v>
       </c>
       <c r="H80" s="7" t="n">
-        <v>23.4</v>
+        <v>46.5</v>
       </c>
       <c r="I80" s="7" t="n">
         <v>0.5</v>
       </c>
       <c r="J80" s="7" t="n">
-        <v>0.5</v>
+        <v>0.92</v>
       </c>
       <c r="K80" s="7" t="n">
         <v>1</v>
@@ -11257,7 +11253,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>shot.dart.A6</t>
+          <t>shot.dart.A5</t>
         </is>
       </c>
       <c r="B81" s="9" t="inlineStr">
@@ -11267,7 +11263,7 @@
       </c>
       <c r="C81" s="9" t="inlineStr">
         <is>
-          <t>投掷物「重罐点名」6 级：双层底座 + 陨石</t>
+          <t>投掷物「重罐点名」5 级：手雷</t>
         </is>
       </c>
       <c r="D81" s="9" t="inlineStr">
@@ -11277,19 +11273,19 @@
       </c>
       <c r="E81" s="8" t="inlineStr">
         <is>
-          <t>art/shot.dart.A6.png</t>
+          <t>art/shot.dart.A5.png</t>
         </is>
       </c>
       <c r="F81" s="8" t="inlineStr">
         <is>
-          <t>art/shot.dart.A6.json</t>
+          <t>art/shot.dart.A5.json</t>
         </is>
       </c>
       <c r="G81" s="7" t="n">
-        <v>42.9</v>
+        <v>23.4</v>
       </c>
       <c r="H81" s="7" t="n">
-        <v>42.9</v>
+        <v>23.4</v>
       </c>
       <c r="I81" s="7" t="n">
         <v>0.5</v>
@@ -11314,17 +11310,17 @@
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
-          <t>fx.drone</t>
+          <t>shot.dart.A6</t>
         </is>
       </c>
       <c r="B82" s="9" t="inlineStr">
         <is>
-          <t>特效</t>
+          <t>子弹</t>
         </is>
       </c>
       <c r="C82" s="9" t="inlineStr">
         <is>
-          <t>鞋盒无人机送货飞行（fly 循环，pivot 在机身中心）</t>
+          <t>投掷物「重罐点名」6 级：双层底座 + 陨石</t>
         </is>
       </c>
       <c r="D82" s="9" t="inlineStr">
@@ -11334,19 +11330,19 @@
       </c>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t>art/fx.drone.png</t>
+          <t>art/shot.dart.A6.png</t>
         </is>
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t>art/fx.drone.json</t>
+          <t>art/shot.dart.A6.json</t>
         </is>
       </c>
       <c r="G82" s="7" t="n">
-        <v>48.9</v>
+        <v>42.9</v>
       </c>
       <c r="H82" s="7" t="n">
-        <v>33.2</v>
+        <v>42.9</v>
       </c>
       <c r="I82" s="7" t="n">
         <v>0.5</v>
@@ -11368,65 +11364,122 @@
         <v/>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="10" t="inlineStr">
-        <is>
-          <t>※ 图片地址填公开可访问的 https:// 链接（PNG / WebP，透明背景）；也可以不填，直接在游戏页面点「导入美术图片」，把文件名改成资源编号（如 tower.dart.png）一次选多张。</t>
-        </is>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>fx.drone</t>
+        </is>
+      </c>
+      <c r="B83" s="9" t="inlineStr">
+        <is>
+          <t>特效</t>
+        </is>
+      </c>
+      <c r="C83" s="9" t="inlineStr">
+        <is>
+          <t>鞋盒无人机送货飞行（fly 循环，pivot 在机身中心）</t>
+        </is>
+      </c>
+      <c r="D83" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="E83" s="8" t="inlineStr">
+        <is>
+          <t>art/fx.drone.png</t>
+        </is>
+      </c>
+      <c r="F83" s="8" t="inlineStr">
+        <is>
+          <t>art/fx.drone.json</t>
+        </is>
+      </c>
+      <c r="G83" s="7" t="n">
+        <v>48.9</v>
+      </c>
+      <c r="H83" s="7" t="n">
+        <v>33.2</v>
+      </c>
+      <c r="I83" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J83" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="K83" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="L83" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M83" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N83" s="9">
+        <f>IF(K83&gt;1,K83*G83*3&amp;" × "&amp;H83*3&amp;"（"&amp;K83&amp;" 帧横排）",G83*3&amp;" × "&amp;H83*3)</f>
+        <v/>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>※ 游戏内宽高以 360 × 600 的画布为单位；出图按 3 倍像素（见最后一列），游戏会缩放到这里填的尺寸。</t>
+          <t>※ 图片地址填公开可访问的 https:// 链接（PNG / WebP，透明背景）；也可以不填，直接在游戏页面点「导入美术图片」，把文件名改成资源编号（如 tower.dart.png）一次选多张。</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
         <is>
-          <t>※ 锚点是图片里对齐游戏坐标的那一点：0,0 = 左上角，0.5,1 = 底边中点（跑者、装置用脚底中点）。</t>
+          <t>※ 游戏内宽高以 360 × 600 的画布为单位；出图按 3 倍像素（见最后一列），游戏会缩放到这里填的尺寸。</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>※ 帧数 &gt; 1 时，图片是横向排开的序列帧（每帧等宽），按帧率循环播放。跑者、Boss 统一画成「侧面向右跑」，向左时游戏自动水平翻转。</t>
+          <t>※ 锚点是图片里对齐游戏坐标的那一点：0,0 = 左上角，0.5,1 = 底边中点（跑者、装置用脚底中点）。</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
         <is>
-          <t>※ 装置变种图 tower.xxx.A3 / A6（B、C 同理）：该路线成为主路线并升到 3 级 / 6 级时替换基础图；没给就往下找，最后用基础图。导入时文件名里的装置也可以写 can / banana / sprinkler / drone / speaker / chill。</t>
+          <t>※ 帧数 &gt; 1 时，图片是横向排开的序列帧（每帧等宽），按帧率循环播放。跑者、Boss 统一画成「侧面向右跑」，向左时游戏自动水平翻转。</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>※ 动画：PNG 精灵图 + 同名 JSON（Aseprite「导出精灵图」勾选 JSON Data，或 TexturePacker JSON）。动画段用 Tag：idle 待机、fire 发射、build 放置、fly 子弹飞行、hit 命中；再用 1 帧的 release Tag 标出子弹离手的那一帧。用 Slice 标点：pivot 脚底 / 中心，muzzle 子弹出手点。导入时把 PNG 和 JSON 一起选上即可，或在「动画 JSON 地址」填链接。</t>
+          <t>※ 装置变种图 tower.xxx.A3 / A6（B、C 同理）：该路线成为主路线并升到 3 级 / 6 级时替换基础图；没给就往下找，最后用基础图。导入时文件名里的装置也可以写 can / banana / sprinkler / drone / speaker / chill。</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
         <is>
-          <t>※ 子弹只画外观：fly 画朝右，游戏沿弹道自动旋转；弹道类型、速度、抛物线高度在「弹道」表里调。</t>
+          <t>※ 动画：PNG 精灵图 + 同名 JSON（Aseprite「导出精灵图」勾选 JSON Data，或 TexturePacker JSON）。动画段用 Tag：idle 待机、fire 发射、build 放置、fly 子弹飞行、hit 命中；再用 1 帧的 release Tag 标出子弹离手的那一帧。用 Slice 标点：pivot 脚底 / 中心，muzzle 子弹出手点。导入时把 PNG 和 JSON 一起选上即可，或在「动画 JSON 地址」填链接。</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
+          <t>※ 子弹只画外观：fly 画朝右，游戏沿弹道自动旋转；弹道类型、速度、抛物线高度在「弹道」表里调。</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="10" t="inlineStr">
+        <is>
           <t>※ 优先级：P1 样板关（先画这些就能完整玩一张图）→ P2 → P3。</t>
         </is>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="M3:M82" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="M3:M83" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"0,1"</formula1>
     </dataValidation>
   </dataValidations>
@@ -11699,7 +11752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D304"/>
+  <dimension ref="A1:D303"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -11777,22 +11830,22 @@
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>6 种装置：易拉罐投手（单体）、香蕉皮投手（范围滑倒）、洒水器（减速、冻结）、鞋盒无人机（全图空投）、广场舞音响（神曲连锁传播）、宝石发射器（红黄蓝三种宝石）。每种 3 条路线、每条 5 级；主路线可升满，次路线最多 2 级。</t>
+          <t>6 种装置 + 矿机：易拉罐投手（单体）、香蕉皮投手（跑道陷阱、滑倒）、洒水车（会自己开，减速、冻结）、鞋盒无人机（全图空投）、广场舞音响（神曲连锁传播）、休闲诱惑站（把跑者留住）；矿机负责挣钱。每种 3 条路线，最多点 2 条；先到 3 级的成为主路线，可一直升到 6 级。</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>6 种装置：易拉罐投手（单体）、香蕉皮投手（范围滑倒）、洒水器（减速、冻结）、鞋盒无人机（全图空投）、广场舞音响（神曲连锁传播）、宝石发射器（红黄蓝三种宝石）。每种 3 条路线、每条 5 级；主路线可升满，次路线最多 2 级。</t>
+          <t>6 种装置 + 矿机：易拉罐投手（单体）、香蕉皮投手（跑道陷阱、滑倒）、洒水车（会自己开，减速、冻结）、鞋盒无人机（全图空投）、广场舞音响（神曲连锁传播）、休闲诱惑站（把跑者留住）；矿机负责挣钱。每种 3 条路线，最多点 2 条；先到 3 级的成为主路线，可一直升到 6 级。</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>6 devices: Can Thrower (single target), Banana Peeler (area slip), Sprinkler (slow, freeze), Shoebox Drone (map-wide drop), Dance Speaker (chain earworm), Gem Launcher (ruby, topaz, sapphire). Each has 3 paths of 5 tiers; the main path can max out, the secondary stops at tier 2.</t>
+          <t>6 devices plus the miner: Can Thrower (single target), Banana Peeler (track traps, slips), Sprinkler Truck (drives itself; slows, freezes), Shoebox Drone (map-wide drops), Dance Speaker (chain earworm), Chill Spot (holds runners up); the miner earns money. Each has 3 paths and you can take 2; the first to tier 3 becomes the main path and goes up to tier 6.</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>6 dispositifs : Lanceur de canettes (cible unique), Lanceur de peaux de banane (glissade de zone), Arroseur (ralentit, gèle), Drone à boîtes (largage sur toute la carte), Enceinte de danse (tube viral en chaîne), Lance-gemmes (rubis, topaze, saphir). Chacun a 3 voies de 5 niveaux ; la voie principale peut être maximisée, la secondaire s’arrête au niveau 2.</t>
+          <t>6 dispositifs plus le Mineur : Lanceur de canettes (cible unique), Lanceur de peaux de banane (pièges sur la piste, glissades), Camion arroseur (roule tout seul ; ralentit, gèle), Drone à boîtes (largages sur toute la carte), Enceinte de danse (tube viral en chaîne), Coin détente (retient les coureurs) ; le Mineur rapporte de l’argent. Chacun a 3 voies, on peut en prendre 2 ; la première au niveau 3 devient la voie principale et monte jusqu’au niveau 6.</t>
         </is>
       </c>
     </row>
@@ -13163,66 +13216,66 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>次路线</t>
+          <t>每波结束开启神秘箱三选一：宝石、GST 红包、GMT 质押、MOOAR 折扣、Gas Hero 毒气、升级卷轴、创世鞋等。局内 GST 只是关卡内货币，不和任何真实资产挂钩。</t>
         </is>
       </c>
       <c r="B67" s="8" t="inlineStr">
         <is>
-          <t>次路线</t>
+          <t>每波结束开启神秘箱三选一：宝石、GST 红包、GMT 质押、MOOAR 折扣、Gas Hero 毒气、升级卷轴、创世鞋等。局内 GST 只是关卡内货币，不和任何真实资产挂钩。</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>After each wave, open a Mystery Box and pick 1 of 3: gems, GST Red Packets, GMT Staking, MOOAR Discount, Gas Hero Gas, Level-up Scrolls, Genesis Sneakers and more. In-run GST is a level-only currency and is not tied to any real asset.</t>
         </is>
       </c>
       <c r="D67" s="8" t="inlineStr">
         <is>
-          <t>Secondaire</t>
+          <t>Après chaque vague, ouvre une Mystery Box et choisis 1 carte sur 3 : gemmes, Enveloppes GST, Staking GMT, Remise MOOAR, Gaz Gas Hero, Parchemins, Sneakers Genesis, etc. Le GST de la partie est une monnaie de niveau, sans lien avec un actif réel.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="6" t="inlineStr">
         <is>
-          <t>每波结束开启神秘箱三选一：宝石、GST 红包、GMT 质押、MOOAR 折扣、Gas Hero 毒气、升级卷轴、创世鞋等。局内 GST 只是关卡内货币，不和任何真实资产挂钩。</t>
+          <t>波次</t>
         </is>
       </c>
       <c r="B68" s="8" t="inlineStr">
         <is>
-          <t>每波结束开启神秘箱三选一：宝石、GST 红包、GMT 质押、MOOAR 折扣、Gas Hero 毒气、升级卷轴、创世鞋等。局内 GST 只是关卡内货币，不和任何真实资产挂钩。</t>
+          <t>波次</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t>After each wave, open a Mystery Box and pick 1 of 3: gems, GST Red Packets, GMT Staking, MOOAR Discount, Gas Hero Gas, Level-up Scrolls, Genesis Sneakers and more. In-run GST is a level-only currency and is not tied to any real asset.</t>
+          <t>Wave</t>
         </is>
       </c>
       <c r="D68" s="8" t="inlineStr">
         <is>
-          <t>Après chaque vague, ouvre une Mystery Box et choisis 1 carte sur 3 : gemmes, Enveloppes GST, Staking GMT, Remise MOOAR, Gaz Gas Hero, Parchemins, Sneakers Genesis, etc. Le GST de la partie est une monnaie de niveau, sans lien avec un actif réel.</t>
+          <t>Vague</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>波次</t>
+          <t>活动范围</t>
         </is>
       </c>
       <c r="B69" s="8" t="inlineStr">
         <is>
-          <t>波次</t>
+          <t>活动范围</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>Wave</t>
+          <t>Patrol</t>
         </is>
       </c>
       <c r="D69" s="8" t="inlineStr">
         <is>
-          <t>Vague</t>
+          <t>Patrouille</t>
         </is>
       </c>
     </row>
@@ -15935,2425 +15988,2403 @@
     <row r="193">
       <c r="A193" s="6" t="inlineStr">
         <is>
-          <t>宝石发射器</t>
+          <t>红宝石</t>
         </is>
       </c>
       <c r="B193" s="8" t="inlineStr">
         <is>
-          <t>宝石发射器</t>
+          <t>红宝石</t>
         </is>
       </c>
       <c r="C193" s="8" t="inlineStr">
         <is>
-          <t>Gem Launcher</t>
+          <t>Ruby</t>
         </is>
       </c>
       <c r="D193" s="8" t="inlineStr">
         <is>
-          <t>Lance-gemmes</t>
+          <t>Rubis</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" s="6" t="inlineStr">
         <is>
-          <t>红宝石</t>
+          <t>蓝宝石</t>
         </is>
       </c>
       <c r="B194" s="8" t="inlineStr">
         <is>
-          <t>红宝石</t>
+          <t>蓝宝石</t>
         </is>
       </c>
       <c r="C194" s="8" t="inlineStr">
         <is>
-          <t>Ruby</t>
+          <t>Sapphire</t>
         </is>
       </c>
       <c r="D194" s="8" t="inlineStr">
         <is>
-          <t>Rubis</t>
+          <t>Saphir</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" s="6" t="inlineStr">
         <is>
-          <t>蓝宝石</t>
+          <t>下一级：{x}</t>
         </is>
       </c>
       <c r="B195" s="8" t="inlineStr">
         <is>
-          <t>蓝宝石</t>
+          <t>下一级：{x}</t>
         </is>
       </c>
       <c r="C195" s="8" t="inlineStr">
         <is>
-          <t>Sapphire</t>
+          <t>Next: {x}</t>
         </is>
       </c>
       <c r="D195" s="8" t="inlineStr">
         <is>
-          <t>Saphir</t>
+          <t>Suivant : {x}</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="6" t="inlineStr">
         <is>
-          <t>下一级：{x}</t>
+          <t>这里不能放</t>
         </is>
       </c>
       <c r="B196" s="8" t="inlineStr">
         <is>
-          <t>下一级：{x}</t>
+          <t>这里不能放</t>
         </is>
       </c>
       <c r="C196" s="8" t="inlineStr">
         <is>
-          <t>Next: {x}</t>
+          <t>Can’t build here</t>
         </is>
       </c>
       <c r="D196" s="8" t="inlineStr">
         <is>
-          <t>Suivant : {x}</t>
+          <t>Impossible ici</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="6" t="inlineStr">
         <is>
-          <t>这里不能放</t>
+          <t>取消放置</t>
         </is>
       </c>
       <c r="B197" s="8" t="inlineStr">
         <is>
-          <t>这里不能放</t>
+          <t>取消放置</t>
         </is>
       </c>
       <c r="C197" s="8" t="inlineStr">
         <is>
-          <t>Can’t build here</t>
+          <t>Cancel placing</t>
         </is>
       </c>
       <c r="D197" s="8" t="inlineStr">
         <is>
-          <t>Impossible ici</t>
+          <t>Annuler</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" s="6" t="inlineStr">
         <is>
-          <t>取消放置</t>
+          <t>＋ 放置点 ×{n}</t>
         </is>
       </c>
       <c r="B198" s="8" t="inlineStr">
         <is>
-          <t>取消放置</t>
+          <t>＋ 放置点 ×{n}</t>
         </is>
       </c>
       <c r="C198" s="8" t="inlineStr">
         <is>
-          <t>Cancel placing</t>
+          <t>+ Spot ×{n}</t>
         </is>
       </c>
       <c r="D198" s="8" t="inlineStr">
         <is>
-          <t>Annuler</t>
+          <t>+ Emplacement ×{n}</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" s="6" t="inlineStr">
         <is>
-          <t>＋ 放置点 ×{n}</t>
+          <t>点跑道外的空地，新增一个放置点</t>
         </is>
       </c>
       <c r="B199" s="8" t="inlineStr">
         <is>
-          <t>＋ 放置点 ×{n}</t>
+          <t>点跑道外的空地，新增一个放置点</t>
         </is>
       </c>
       <c r="C199" s="8" t="inlineStr">
         <is>
-          <t>+ Spot ×{n}</t>
+          <t>Tap open ground off the track to add a spot</t>
         </is>
       </c>
       <c r="D199" s="8" t="inlineStr">
         <is>
-          <t>+ Emplacement ×{n}</t>
+          <t>Touche un terrain libre hors piste pour ajouter un emplacement</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" s="6" t="inlineStr">
         <is>
-          <t>点跑道外的空地，新增一个放置点</t>
+          <t>聪</t>
         </is>
       </c>
       <c r="B200" s="8" t="inlineStr">
         <is>
-          <t>点跑道外的空地，新增一个放置点</t>
+          <t>聪</t>
         </is>
       </c>
       <c r="C200" s="8" t="inlineStr">
         <is>
-          <t>Tap open ground off the track to add a spot</t>
+          <t>sats</t>
         </is>
       </c>
       <c r="D200" s="8" t="inlineStr">
         <is>
-          <t>Touche un terrain libre hors piste pour ajouter un emplacement</t>
+          <t>sats</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" s="6" t="inlineStr">
         <is>
-          <t>聪</t>
+          <t>创世纪 · 2008–2010</t>
         </is>
       </c>
       <c r="B201" s="8" t="inlineStr">
         <is>
-          <t>聪</t>
+          <t>创世纪 · 2008–2010</t>
         </is>
       </c>
       <c r="C201" s="8" t="inlineStr">
         <is>
-          <t>sats</t>
+          <t>Genesis · 2008–2010</t>
         </is>
       </c>
       <c r="D201" s="8" t="inlineStr">
         <is>
-          <t>sats</t>
+          <t>Genèse · 2008–2010</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" s="6" t="inlineStr">
         <is>
-          <t>创世纪 · 2008–2010</t>
+          <t>组合</t>
         </is>
       </c>
       <c r="B202" s="8" t="inlineStr">
         <is>
-          <t>创世纪 · 2008–2010</t>
+          <t>组合</t>
         </is>
       </c>
       <c r="C202" s="8" t="inlineStr">
         <is>
-          <t>Genesis · 2008–2010</t>
+          <t>Combos</t>
         </is>
       </c>
       <c r="D202" s="8" t="inlineStr">
         <is>
-          <t>Genèse · 2008–2010</t>
+          <t>Combos</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" s="6" t="inlineStr">
         <is>
-          <t>组合</t>
+          <t>重试</t>
         </is>
       </c>
       <c r="B203" s="8" t="inlineStr">
         <is>
-          <t>组合</t>
+          <t>重试</t>
         </is>
       </c>
       <c r="C203" s="8" t="inlineStr">
         <is>
-          <t>Combos</t>
+          <t>Retry</t>
         </is>
       </c>
       <c r="D203" s="8" t="inlineStr">
         <is>
-          <t>Combos</t>
+          <t>Réessayer</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" s="6" t="inlineStr">
         <is>
-          <t>重试</t>
+          <t>STEPN 跑者掉进区块链时光隧道，跟着比特币走过最初的三年。</t>
         </is>
       </c>
       <c r="B204" s="8" t="inlineStr">
         <is>
-          <t>重试</t>
+          <t>STEPN 跑者掉进区块链时光隧道，跟着比特币走过最初的三年。</t>
         </is>
       </c>
       <c r="C204" s="8" t="inlineStr">
         <is>
-          <t>Retry</t>
+          <t>A STEPN runner falls into a blockchain time tunnel and lives through bitcoin’s first three years.</t>
         </is>
       </c>
       <c r="D204" s="8" t="inlineStr">
         <is>
-          <t>Réessayer</t>
+          <t>Un coureur STEPN tombe dans un tunnel temporel blockchain et vit les trois premières années du bitcoin.</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" s="6" t="inlineStr">
         <is>
-          <t>STEPN 跑者掉进区块链时光隧道，跟着比特币走过最初的三年。</t>
+          <t>累计积分 {n}</t>
         </is>
       </c>
       <c r="B205" s="8" t="inlineStr">
         <is>
-          <t>STEPN 跑者掉进区块链时光隧道，跟着比特币走过最初的三年。</t>
+          <t>累计积分 {n}</t>
         </is>
       </c>
       <c r="C205" s="8" t="inlineStr">
         <is>
-          <t>A STEPN runner falls into a blockchain time tunnel and lives through bitcoin’s first three years.</t>
+          <t>Points: {n}</t>
         </is>
       </c>
       <c r="D205" s="8" t="inlineStr">
         <is>
-          <t>Un coureur STEPN tombe dans un tunnel temporel blockchain et vit les trois premières années du bitcoin.</t>
+          <t>Points : {n}</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" s="6" t="inlineStr">
         <is>
-          <t>累计积分 {n}</t>
+          <t>剧情中…</t>
         </is>
       </c>
       <c r="B206" s="8" t="inlineStr">
         <is>
-          <t>累计积分 {n}</t>
+          <t>剧情中…</t>
         </is>
       </c>
       <c r="C206" s="8" t="inlineStr">
         <is>
-          <t>Points: {n}</t>
+          <t>Story…</t>
         </is>
       </c>
       <c r="D206" s="8" t="inlineStr">
         <is>
-          <t>Points : {n}</t>
+          <t>Histoire…</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" s="6" t="inlineStr">
         <is>
-          <t>剧情中…</t>
+          <t>关卡完成</t>
         </is>
       </c>
       <c r="B207" s="8" t="inlineStr">
         <is>
-          <t>剧情中…</t>
+          <t>关卡完成</t>
         </is>
       </c>
       <c r="C207" s="8" t="inlineStr">
         <is>
-          <t>Story…</t>
+          <t>Level complete</t>
         </is>
       </c>
       <c r="D207" s="8" t="inlineStr">
         <is>
-          <t>Histoire…</t>
+          <t>Niveau terminé</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" s="6" t="inlineStr">
         <is>
-          <t>关卡完成</t>
+          <t>再玩一次</t>
         </is>
       </c>
       <c r="B208" s="8" t="inlineStr">
         <is>
-          <t>关卡完成</t>
+          <t>再玩一次</t>
         </is>
       </c>
       <c r="C208" s="8" t="inlineStr">
         <is>
-          <t>Level complete</t>
+          <t>Play again</t>
         </is>
       </c>
       <c r="D208" s="8" t="inlineStr">
         <is>
-          <t>Niveau terminé</t>
+          <t>Rejouer</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" s="6" t="inlineStr">
         <is>
-          <t>再玩一次</t>
+          <t>章节地图</t>
         </is>
       </c>
       <c r="B209" s="8" t="inlineStr">
         <is>
-          <t>再玩一次</t>
+          <t>章节地图</t>
         </is>
       </c>
       <c r="C209" s="8" t="inlineStr">
         <is>
-          <t>Play again</t>
+          <t>Chapter map</t>
         </is>
       </c>
       <c r="D209" s="8" t="inlineStr">
         <is>
-          <t>Rejouer</t>
+          <t>Carte du chapitre</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" s="6" t="inlineStr">
         <is>
-          <t>章节地图</t>
+          <t>第二章 · 敬请期待</t>
         </is>
       </c>
       <c r="B210" s="8" t="inlineStr">
         <is>
-          <t>章节地图</t>
+          <t>第二章 · 敬请期待</t>
         </is>
       </c>
       <c r="C210" s="8" t="inlineStr">
         <is>
-          <t>Chapter map</t>
+          <t>Chapter 2 · coming soon</t>
         </is>
       </c>
       <c r="D210" s="8" t="inlineStr">
         <is>
-          <t>Carte du chapitre</t>
+          <t>Chapitre 2 · bientôt</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" s="6" t="inlineStr">
         <is>
-          <t>第二章 · 敬请期待</t>
+          <t>图鉴</t>
         </is>
       </c>
       <c r="B211" s="8" t="inlineStr">
         <is>
-          <t>第二章 · 敬请期待</t>
+          <t>图鉴</t>
         </is>
       </c>
       <c r="C211" s="8" t="inlineStr">
         <is>
-          <t>Chapter 2 · coming soon</t>
+          <t>Codex</t>
         </is>
       </c>
       <c r="D211" s="8" t="inlineStr">
         <is>
-          <t>Chapitre 2 · bientôt</t>
+          <t>Codex</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" s="6" t="inlineStr">
         <is>
-          <t>图鉴</t>
+          <t>区块高度</t>
         </is>
       </c>
       <c r="B212" s="8" t="inlineStr">
         <is>
-          <t>图鉴</t>
+          <t>区块高度</t>
         </is>
       </c>
       <c r="C212" s="8" t="inlineStr">
         <is>
-          <t>Codex</t>
+          <t>Block height</t>
         </is>
       </c>
       <c r="D212" s="8" t="inlineStr">
         <is>
-          <t>Codex</t>
+          <t>Hauteur</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" s="6" t="inlineStr">
         <is>
-          <t>区块高度</t>
+          <t>区块奖励：选一个，比赛马上继续。</t>
         </is>
       </c>
       <c r="B213" s="8" t="inlineStr">
         <is>
-          <t>区块高度</t>
+          <t>区块奖励：选一个，比赛马上继续。</t>
         </is>
       </c>
       <c r="C213" s="8" t="inlineStr">
         <is>
-          <t>Block height</t>
+          <t>Block reward: pick one and the race resumes.</t>
         </is>
       </c>
       <c r="D213" s="8" t="inlineStr">
         <is>
-          <t>Hauteur</t>
+          <t>Récompense de bloc : choisis-en une et la course reprend.</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" s="6" t="inlineStr">
         <is>
-          <t>区块奖励：选一个，比赛马上继续。</t>
+          <t>选择关卡</t>
         </is>
       </c>
       <c r="B214" s="8" t="inlineStr">
         <is>
-          <t>区块奖励：选一个，比赛马上继续。</t>
+          <t>选择关卡</t>
         </is>
       </c>
       <c r="C214" s="8" t="inlineStr">
         <is>
-          <t>Block reward: pick one and the race resumes.</t>
+          <t>Choose a level</t>
         </is>
       </c>
       <c r="D214" s="8" t="inlineStr">
         <is>
-          <t>Récompense de bloc : choisis-en une et la course reprend.</t>
+          <t>Choisir un niveau</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" s="6" t="inlineStr">
         <is>
-          <t>选择关卡</t>
+          <t>这关还没打出组合，试试把两种状态叠在同一个跑者身上。</t>
         </is>
       </c>
       <c r="B215" s="8" t="inlineStr">
         <is>
-          <t>选择关卡</t>
+          <t>这关还没打出组合，试试把两种状态叠在同一个跑者身上。</t>
         </is>
       </c>
       <c r="C215" s="8" t="inlineStr">
         <is>
-          <t>Choose a level</t>
+          <t>No combos this time. Try stacking two statuses on the same runner.</t>
         </is>
       </c>
       <c r="D215" s="8" t="inlineStr">
         <is>
-          <t>Choisir un niveau</t>
+          <t>Aucun combo cette fois. Essaie de cumuler deux états sur le même coureur.</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" s="6" t="inlineStr">
         <is>
-          <t>这关还没打出组合，试试把两种状态叠在同一个跑者身上。</t>
+          <t>快捷键：空格 开波 · F 切换速度 · 1–7 建造 · Q/W/E 升级 · X 回收 · Esc 取消</t>
         </is>
       </c>
       <c r="B216" s="8" t="inlineStr">
         <is>
-          <t>这关还没打出组合，试试把两种状态叠在同一个跑者身上。</t>
+          <t>快捷键：空格 开波 · F 切换速度 · 1–7 建造 · Q/W/E 升级 · X 回收 · Esc 取消</t>
         </is>
       </c>
       <c r="C216" s="8" t="inlineStr">
         <is>
-          <t>No combos this time. Try stacking two statuses on the same runner.</t>
+          <t>Keys: Space start wave · F speed · 1–7 build · Q/W/E upgrade · X recycle · Esc cancel</t>
         </is>
       </c>
       <c r="D216" s="8" t="inlineStr">
         <is>
-          <t>Aucun combo cette fois. Essaie de cumuler deux états sur le même coureur.</t>
+          <t>Touches : Espace vague · F vitesse · 1–7 construire · Q/W/E améliorer · X recycler · Échap annuler</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" s="6" t="inlineStr">
         <is>
-          <t>快捷键：空格 开波 · F 切换速度 · 1–7 建造 · Q/W/E 升级 · X 回收 · Esc 取消</t>
+          <t>一万枚换两个披萨！</t>
         </is>
       </c>
       <c r="B217" s="8" t="inlineStr">
         <is>
-          <t>快捷键：空格 开波 · F 切换速度 · 1–7 建造 · Q/W/E 升级 · X 回收 · Esc 取消</t>
+          <t>一万枚换两个披萨！</t>
         </is>
       </c>
       <c r="C217" s="8" t="inlineStr">
         <is>
-          <t>Keys: Space start wave · F speed · 1–7 build · Q/W/E upgrade · X recycle · Esc cancel</t>
+          <t>10,000 coins for two pizzas!</t>
         </is>
       </c>
       <c r="D217" s="8" t="inlineStr">
         <is>
-          <t>Touches : Espace vague · F vitesse · 1–7 construire · Q/W/E améliorer · X recycler · Échap annuler</t>
+          <t>10 000 pièces pour deux pizzas !</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" s="6" t="inlineStr">
         <is>
-          <t>一万枚换两个披萨！</t>
+          <t>知识卡</t>
         </is>
       </c>
       <c r="B218" s="8" t="inlineStr">
         <is>
-          <t>一万枚换两个披萨！</t>
+          <t>知识卡</t>
         </is>
       </c>
       <c r="C218" s="8" t="inlineStr">
         <is>
-          <t>10,000 coins for two pizzas!</t>
+          <t>Knowledge</t>
         </is>
       </c>
       <c r="D218" s="8" t="inlineStr">
         <is>
-          <t>10 000 pièces pour deux pizzas !</t>
+          <t>Savoir</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" s="6" t="inlineStr">
         <is>
-          <t>知识卡</t>
+          <t>新组合：{x}！</t>
         </is>
       </c>
       <c r="B219" s="8" t="inlineStr">
         <is>
-          <t>知识卡</t>
+          <t>新组合：{x}！</t>
         </is>
       </c>
       <c r="C219" s="8" t="inlineStr">
         <is>
-          <t>Knowledge</t>
+          <t>New combo: {x}!</t>
         </is>
       </c>
       <c r="D219" s="8" t="inlineStr">
         <is>
-          <t>Savoir</t>
+          <t>Nouveau combo : {x} !</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" s="6" t="inlineStr">
         <is>
-          <t>新组合：{x}！</t>
+          <t>下一关</t>
         </is>
       </c>
       <c r="B220" s="8" t="inlineStr">
         <is>
-          <t>新组合：{x}！</t>
+          <t>下一关</t>
         </is>
       </c>
       <c r="C220" s="8" t="inlineStr">
         <is>
-          <t>New combo: {x}!</t>
+          <t>Next level</t>
         </is>
       </c>
       <c r="D220" s="8" t="inlineStr">
         <is>
-          <t>Nouveau combo : {x} !</t>
+          <t>Niveau suivant</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" s="6" t="inlineStr">
         <is>
-          <t>下一关</t>
+          <t>{n}× 速度</t>
         </is>
       </c>
       <c r="B221" s="8" t="inlineStr">
         <is>
-          <t>下一关</t>
+          <t>{n}× 速度</t>
         </is>
       </c>
       <c r="C221" s="8" t="inlineStr">
         <is>
-          <t>Next level</t>
+          <t>{n}× speed</t>
         </is>
       </c>
       <c r="D221" s="8" t="inlineStr">
         <is>
-          <t>Niveau suivant</t>
+          <t>Vitesse ×{n}</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" s="6" t="inlineStr">
         <is>
-          <t>{n}× 速度</t>
+          <t>区块 #{h} 被别的矿工抢先挖到了</t>
         </is>
       </c>
       <c r="B222" s="8" t="inlineStr">
         <is>
-          <t>{n}× 速度</t>
+          <t>区块 #{h} 被别的矿工抢先挖到了</t>
         </is>
       </c>
       <c r="C222" s="8" t="inlineStr">
         <is>
-          <t>{n}× speed</t>
+          <t>Block #{h} went to another miner</t>
         </is>
       </c>
       <c r="D222" s="8" t="inlineStr">
         <is>
-          <t>Vitesse ×{n}</t>
+          <t>Le bloc #{h} est allé à un autre mineur</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" s="6" t="inlineStr">
         <is>
-          <t>区块 #{h} 被别的矿工抢先挖到了</t>
+          <t>挖到区块</t>
         </is>
       </c>
       <c r="B223" s="8" t="inlineStr">
         <is>
-          <t>区块 #{h} 被别的矿工抢先挖到了</t>
+          <t>挖到区块</t>
         </is>
       </c>
       <c r="C223" s="8" t="inlineStr">
         <is>
-          <t>Block #{h} went to another miner</t>
+          <t>Blocks mined</t>
         </is>
       </c>
       <c r="D223" s="8" t="inlineStr">
         <is>
-          <t>Le bloc #{h} est allé à un autre mineur</t>
+          <t>Blocs minés</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" s="6" t="inlineStr">
         <is>
-          <t>挖到区块</t>
+          <t>本关触发的组合</t>
         </is>
       </c>
       <c r="B224" s="8" t="inlineStr">
         <is>
-          <t>挖到区块</t>
+          <t>本关触发的组合</t>
         </is>
       </c>
       <c r="C224" s="8" t="inlineStr">
         <is>
-          <t>Blocks mined</t>
+          <t>Combos this level</t>
         </is>
       </c>
       <c r="D224" s="8" t="inlineStr">
         <is>
-          <t>Blocs minés</t>
+          <t>Combos de ce niveau</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" s="6" t="inlineStr">
         <is>
-          <t>本关触发的组合</t>
+          <t>组合：{x}</t>
         </is>
       </c>
       <c r="B225" s="8" t="inlineStr">
         <is>
-          <t>本关触发的组合</t>
+          <t>组合：{x}</t>
         </is>
       </c>
       <c r="C225" s="8" t="inlineStr">
         <is>
-          <t>Combos this level</t>
+          <t>Combos: {x}</t>
         </is>
       </c>
       <c r="D225" s="8" t="inlineStr">
         <is>
-          <t>Combos de ce niveau</t>
+          <t>Combos : {x}</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" s="6" t="inlineStr">
         <is>
-          <t>组合：{x}</t>
+          <t>修复版本上线，溢出的币被回滚</t>
         </is>
       </c>
       <c r="B226" s="8" t="inlineStr">
         <is>
-          <t>组合：{x}</t>
+          <t>修复版本上线，溢出的币被回滚</t>
         </is>
       </c>
       <c r="C226" s="8" t="inlineStr">
         <is>
-          <t>Combos: {x}</t>
+          <t>The fix is live; the overflowed coins are rolled back</t>
         </is>
       </c>
       <c r="D226" s="8" t="inlineStr">
         <is>
-          <t>Combos : {x}</t>
+          <t>Le correctif est en ligne ; les pièces en trop sont annulées</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" s="6" t="inlineStr">
         <is>
-          <t>修复版本上线，溢出的币被回滚</t>
+          <t>还没触发过。试试把这两种状态叠在同一个跑者身上。</t>
         </is>
       </c>
       <c r="B227" s="8" t="inlineStr">
         <is>
-          <t>修复版本上线，溢出的币被回滚</t>
+          <t>还没触发过。试试把这两种状态叠在同一个跑者身上。</t>
         </is>
       </c>
       <c r="C227" s="8" t="inlineStr">
         <is>
-          <t>The fix is live; the overflowed coins are rolled back</t>
+          <t>Not triggered yet. Try stacking these two statuses on one runner.</t>
         </is>
       </c>
       <c r="D227" s="8" t="inlineStr">
         <is>
-          <t>Le correctif est en ligne ; les pièces en trop sont annulées</t>
+          <t>Pas encore déclenché. Cumule ces deux états sur un coureur.</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" s="6" t="inlineStr">
         <is>
-          <t>还没触发过。试试把这两种状态叠在同一个跑者身上。</t>
+          <t>出块！#{h}</t>
         </is>
       </c>
       <c r="B228" s="8" t="inlineStr">
         <is>
-          <t>还没触发过。试试把这两种状态叠在同一个跑者身上。</t>
+          <t>出块！#{h}</t>
         </is>
       </c>
       <c r="C228" s="8" t="inlineStr">
         <is>
-          <t>Not triggered yet. Try stacking these two statuses on one runner.</t>
+          <t>Block! #{h}</t>
         </is>
       </c>
       <c r="D228" s="8" t="inlineStr">
         <is>
-          <t>Pas encore déclenché. Cumule ces deux états sur un coureur.</t>
+          <t>Bloc ! #{h}</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" s="6" t="inlineStr">
         <is>
-          <t>出块！#{h}</t>
+          <t>挖到区块 #{h}！</t>
         </is>
       </c>
       <c r="B229" s="8" t="inlineStr">
         <is>
-          <t>出块！#{h}</t>
+          <t>挖到区块 #{h}！</t>
         </is>
       </c>
       <c r="C229" s="8" t="inlineStr">
         <is>
-          <t>Block! #{h}</t>
+          <t>Mined block #{h}!</t>
         </is>
       </c>
       <c r="D229" s="8" t="inlineStr">
         <is>
-          <t>Bloc ! #{h}</t>
+          <t>Bloc #{h} miné !</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" s="6" t="inlineStr">
         <is>
-          <t>挖到区块 #{h}！</t>
+          <t>披萨跑者冲出来了</t>
         </is>
       </c>
       <c r="B230" s="8" t="inlineStr">
         <is>
-          <t>挖到区块 #{h}！</t>
+          <t>披萨跑者冲出来了</t>
         </is>
       </c>
       <c r="C230" s="8" t="inlineStr">
         <is>
-          <t>Mined block #{h}!</t>
+          <t>Pizza runners incoming</t>
         </is>
       </c>
       <c r="D230" s="8" t="inlineStr">
         <is>
-          <t>Bloc #{h} miné !</t>
+          <t>Les coureurs-pizza arrivent</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" s="6" t="inlineStr">
         <is>
-          <t>披萨跑者冲出来了</t>
+          <t>重抽 · {n} 聪</t>
         </is>
       </c>
       <c r="B231" s="8" t="inlineStr">
         <is>
-          <t>披萨跑者冲出来了</t>
+          <t>重抽 · {n} 聪</t>
         </is>
       </c>
       <c r="C231" s="8" t="inlineStr">
         <is>
-          <t>Pizza runners incoming</t>
+          <t>Reroll · {n} sats</t>
         </is>
       </c>
       <c r="D231" s="8" t="inlineStr">
         <is>
-          <t>Les coureurs-pizza arrivent</t>
+          <t>Relancer · {n} sats</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" s="6" t="inlineStr">
         <is>
-          <t>重抽 · {n} 聪</t>
+          <t>继续 ▶</t>
         </is>
       </c>
       <c r="B232" s="8" t="inlineStr">
         <is>
-          <t>重抽 · {n} 聪</t>
+          <t>继续 ▶</t>
         </is>
       </c>
       <c r="C232" s="8" t="inlineStr">
         <is>
-          <t>Reroll · {n} sats</t>
+          <t>Next ▶</t>
         </is>
       </c>
       <c r="D232" s="8" t="inlineStr">
         <is>
-          <t>Relancer · {n} sats</t>
+          <t>Suite ▶</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" s="6" t="inlineStr">
         <is>
-          <t>继续 ▶</t>
+          <t>收入图鉴</t>
         </is>
       </c>
       <c r="B233" s="8" t="inlineStr">
         <is>
-          <t>继续 ▶</t>
+          <t>收入图鉴</t>
         </is>
       </c>
       <c r="C233" s="8" t="inlineStr">
         <is>
-          <t>Next ▶</t>
+          <t>Add to codex</t>
         </is>
       </c>
       <c r="D233" s="8" t="inlineStr">
         <is>
-          <t>Suite ▶</t>
+          <t>Ajouter au codex</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" s="6" t="inlineStr">
         <is>
-          <t>收入图鉴</t>
+          <t>返回章节地图</t>
         </is>
       </c>
       <c r="B234" s="8" t="inlineStr">
         <is>
-          <t>收入图鉴</t>
+          <t>返回章节地图</t>
         </is>
       </c>
       <c r="C234" s="8" t="inlineStr">
         <is>
-          <t>Add to codex</t>
+          <t>Back to chapter map</t>
         </is>
       </c>
       <c r="D234" s="8" t="inlineStr">
         <is>
-          <t>Ajouter au codex</t>
+          <t>Retour à la carte</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" s="6" t="inlineStr">
         <is>
-          <t>返回章节地图</t>
+          <t>跳过</t>
         </is>
       </c>
       <c r="B235" s="8" t="inlineStr">
         <is>
-          <t>返回章节地图</t>
+          <t>跳过</t>
         </is>
       </c>
       <c r="C235" s="8" t="inlineStr">
         <is>
-          <t>Back to chapter map</t>
+          <t>Skip</t>
         </is>
       </c>
       <c r="D235" s="8" t="inlineStr">
         <is>
-          <t>Retour à la carte</t>
+          <t>Passer</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" s="6" t="inlineStr">
         <is>
-          <t>跳过</t>
+          <t>经典模式</t>
         </is>
       </c>
       <c r="B236" s="8" t="inlineStr">
         <is>
-          <t>跳过</t>
+          <t>经典模式</t>
         </is>
       </c>
       <c r="C236" s="8" t="inlineStr">
         <is>
-          <t>Skip</t>
+          <t>Classic mode</t>
         </is>
       </c>
       <c r="D236" s="8" t="inlineStr">
         <is>
-          <t>Passer</t>
+          <t>Mode classique</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" s="6" t="inlineStr">
         <is>
-          <t>经典模式</t>
+          <t>开始！</t>
         </is>
       </c>
       <c r="B237" s="8" t="inlineStr">
         <is>
-          <t>经典模式</t>
+          <t>开始！</t>
         </is>
       </c>
       <c r="C237" s="8" t="inlineStr">
         <is>
-          <t>Classic mode</t>
+          <t>Go!</t>
         </is>
       </c>
       <c r="D237" s="8" t="inlineStr">
         <is>
-          <t>Mode classique</t>
+          <t>C’est parti !</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" s="6" t="inlineStr">
         <is>
-          <t>开始！</t>
+          <t>算力 {h} · 出块奖励 +{b}%</t>
         </is>
       </c>
       <c r="B238" s="8" t="inlineStr">
         <is>
-          <t>开始！</t>
+          <t>算力 {h} · 出块奖励 +{b}%</t>
         </is>
       </c>
       <c r="C238" s="8" t="inlineStr">
         <is>
-          <t>Go!</t>
+          <t>Hash {h} · block reward +{b}%</t>
         </is>
       </c>
       <c r="D238" s="8" t="inlineStr">
         <is>
-          <t>C’est parti !</t>
+          <t>Puissance {h} · récompense +{b} %</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" s="6" t="inlineStr">
         <is>
-          <t>算力 {h} · 出块奖励 +{b}%</t>
+          <t>全网每隔十几秒出一个区块，你的算力占全网的比例，就是抢到它的几率。挖到区块：得聪，再开一次三选一。</t>
         </is>
       </c>
       <c r="B239" s="8" t="inlineStr">
         <is>
-          <t>算力 {h} · 出块奖励 +{b}%</t>
+          <t>全网每隔十几秒出一个区块，你的算力占全网的比例，就是抢到它的几率。挖到区块：得聪，再开一次三选一。</t>
         </is>
       </c>
       <c r="C239" s="8" t="inlineStr">
         <is>
-          <t>Hash {h} · block reward +{b}%</t>
+          <t>The network makes a block every dozen seconds or so. Your share of total hash power is your chance of winning it. Win a block: sats plus a pick-one-of-three.</t>
         </is>
       </c>
       <c r="D239" s="8" t="inlineStr">
         <is>
-          <t>Puissance {h} · récompense +{b} %</t>
+          <t>Le réseau produit un bloc toutes les quinze secondes environ. Ta part de la puissance totale est ta chance de le gagner. Bloc gagné : des sats et un choix parmi trois.</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" s="6" t="inlineStr">
         <is>
-          <t>全网每隔十几秒出一个区块，你的算力占全网的比例，就是抢到它的几率。挖到区块：得聪，再开一次三选一。</t>
+          <t>出块几率</t>
         </is>
       </c>
       <c r="B240" s="8" t="inlineStr">
         <is>
-          <t>全网每隔十几秒出一个区块，你的算力占全网的比例，就是抢到它的几率。挖到区块：得聪，再开一次三选一。</t>
+          <t>出块几率</t>
         </is>
       </c>
       <c r="C240" s="8" t="inlineStr">
         <is>
-          <t>The network makes a block every dozen seconds or so. Your share of total hash power is your chance of winning it. Win a block: sats plus a pick-one-of-three.</t>
+          <t>Win chance</t>
         </is>
       </c>
       <c r="D240" s="8" t="inlineStr">
         <is>
-          <t>Le réseau produit un bloc toutes les quinze secondes environ. Ta part de la puissance totale est ta chance de le gagner. Bloc gagné : des sats et un choix parmi trois.</t>
+          <t>Chance</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" s="6" t="inlineStr">
         <is>
-          <t>出块几率</t>
+          <t>软分叉！</t>
         </is>
       </c>
       <c r="B241" s="8" t="inlineStr">
         <is>
-          <t>出块几率</t>
+          <t>软分叉！</t>
         </is>
       </c>
       <c r="C241" s="8" t="inlineStr">
         <is>
-          <t>Win chance</t>
+          <t>Soft fork!</t>
         </is>
       </c>
       <c r="D241" s="8" t="inlineStr">
         <is>
-          <t>Chance</t>
+          <t>Soft fork !</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" s="6" t="inlineStr">
         <is>
-          <t>软分叉！</t>
+          <t>原型阶段的链下积分，没有任何实际价值</t>
         </is>
       </c>
       <c r="B242" s="8" t="inlineStr">
         <is>
-          <t>软分叉！</t>
+          <t>原型阶段的链下积分，没有任何实际价值</t>
         </is>
       </c>
       <c r="C242" s="8" t="inlineStr">
         <is>
-          <t>Soft fork!</t>
+          <t>off-chain prototype points with no real-world value</t>
         </is>
       </c>
       <c r="D242" s="8" t="inlineStr">
         <is>
-          <t>Soft fork !</t>
+          <t>points hors chaîne du prototype, sans valeur réelle</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" s="6" t="inlineStr">
         <is>
-          <t>原型阶段的链下积分，没有任何实际价值</t>
+          <t>你的算力</t>
         </is>
       </c>
       <c r="B243" s="8" t="inlineStr">
         <is>
-          <t>原型阶段的链下积分，没有任何实际价值</t>
+          <t>你的算力</t>
         </is>
       </c>
       <c r="C243" s="8" t="inlineStr">
         <is>
-          <t>off-chain prototype points with no real-world value</t>
+          <t>Your hash</t>
         </is>
       </c>
       <c r="D243" s="8" t="inlineStr">
         <is>
-          <t>points hors chaîne du prototype, sans valeur réelle</t>
+          <t>Ta puissance</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" s="6" t="inlineStr">
         <is>
-          <t>你的算力</t>
+          <t>挖到的聪</t>
         </is>
       </c>
       <c r="B244" s="8" t="inlineStr">
         <is>
-          <t>你的算力</t>
+          <t>挖到的聪</t>
         </is>
       </c>
       <c r="C244" s="8" t="inlineStr">
         <is>
-          <t>Your hash</t>
+          <t>Sats mined</t>
         </is>
       </c>
       <c r="D244" s="8" t="inlineStr">
         <is>
-          <t>Ta puissance</t>
+          <t>Sats minés</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" s="6" t="inlineStr">
         <is>
-          <t>挖到的聪</t>
+          <t>全网算力</t>
         </is>
       </c>
       <c r="B245" s="8" t="inlineStr">
         <is>
-          <t>挖到的聪</t>
+          <t>全网算力</t>
         </is>
       </c>
       <c r="C245" s="8" t="inlineStr">
         <is>
-          <t>Sats mined</t>
+          <t>Network hash</t>
         </is>
       </c>
       <c r="D245" s="8" t="inlineStr">
         <is>
-          <t>Sats minés</t>
+          <t>Puissance réseau</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" s="6" t="inlineStr">
         <is>
-          <t>全网算力</t>
+          <t>已挖到</t>
         </is>
       </c>
       <c r="B246" s="8" t="inlineStr">
         <is>
-          <t>全网算力</t>
+          <t>已挖到</t>
         </is>
       </c>
       <c r="C246" s="8" t="inlineStr">
         <is>
-          <t>Network hash</t>
+          <t>Won</t>
         </is>
       </c>
       <c r="D246" s="8" t="inlineStr">
         <is>
-          <t>Puissance réseau</t>
+          <t>Gagnés</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" s="6" t="inlineStr">
         <is>
-          <t>已挖到</t>
+          <t>下个区块</t>
         </is>
       </c>
       <c r="B247" s="8" t="inlineStr">
         <is>
-          <t>已挖到</t>
+          <t>下个区块</t>
         </is>
       </c>
       <c r="C247" s="8" t="inlineStr">
         <is>
-          <t>Won</t>
+          <t>Next block</t>
         </is>
       </c>
       <c r="D247" s="8" t="inlineStr">
         <is>
-          <t>Gagnés</t>
+          <t>Prochain bloc</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" s="6" t="inlineStr">
         <is>
-          <t>下个区块</t>
+          <t>剩余生命</t>
         </is>
       </c>
       <c r="B248" s="8" t="inlineStr">
         <is>
-          <t>下个区块</t>
+          <t>剩余生命</t>
         </is>
       </c>
       <c r="C248" s="8" t="inlineStr">
         <is>
-          <t>Next block</t>
+          <t>Lives left</t>
         </is>
       </c>
       <c r="D248" s="8" t="inlineStr">
         <is>
-          <t>Prochain bloc</t>
+          <t>Vies restantes</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" s="6" t="inlineStr">
         <is>
-          <t>剩余生命</t>
+          <t>快捷键 Q / W / E 升级，X 回收</t>
         </is>
       </c>
       <c r="B249" s="8" t="inlineStr">
         <is>
-          <t>剩余生命</t>
+          <t>快捷键 Q / W / E 升级，X 回收</t>
         </is>
       </c>
       <c r="C249" s="8" t="inlineStr">
         <is>
-          <t>Lives left</t>
+          <t>Keys Q / W / E upgrade, X recycles</t>
         </is>
       </c>
       <c r="D249" s="8" t="inlineStr">
         <is>
-          <t>Vies restantes</t>
+          <t>Touches Q / W / E améliorer, X recycler</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" s="6" t="inlineStr">
         <is>
-          <t>快捷键 Q / W / E 升级，X 回收</t>
+          <t>整数溢出！</t>
         </is>
       </c>
       <c r="B250" s="8" t="inlineStr">
         <is>
-          <t>快捷键 Q / W / E 升级，X 回收</t>
+          <t>整数溢出！</t>
         </is>
       </c>
       <c r="C250" s="8" t="inlineStr">
         <is>
-          <t>Keys Q / W / E upgrade, X recycles</t>
+          <t>Integer overflow!</t>
         </is>
       </c>
       <c r="D250" s="8" t="inlineStr">
         <is>
-          <t>Touches Q / W / E améliorer, X recycler</t>
+          <t>Dépassement d’entier !</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" s="6" t="inlineStr">
         <is>
-          <t>整数溢出！</t>
+          <t>第一章</t>
         </is>
       </c>
       <c r="B251" s="8" t="inlineStr">
         <is>
-          <t>整数溢出！</t>
+          <t>第一章</t>
         </is>
       </c>
       <c r="C251" s="8" t="inlineStr">
         <is>
-          <t>Integer overflow!</t>
+          <t>Chapter 1</t>
         </is>
       </c>
       <c r="D251" s="8" t="inlineStr">
         <is>
-          <t>Dépassement d’entier !</t>
+          <t>Chapitre 1</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" s="6" t="inlineStr">
         <is>
-          <t>第一章</t>
+          <t>通关「{x}」解锁</t>
         </is>
       </c>
       <c r="B252" s="8" t="inlineStr">
         <is>
-          <t>第一章</t>
+          <t>通关「{x}」解锁</t>
         </is>
       </c>
       <c r="C252" s="8" t="inlineStr">
         <is>
-          <t>Chapter 1</t>
+          <t>Clear “{x}” to unlock</t>
         </is>
       </c>
       <c r="D252" s="8" t="inlineStr">
         <is>
-          <t>Chapitre 1</t>
+          <t>Termine « {x} » pour débloquer</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" s="6" t="inlineStr">
         <is>
-          <t>通关「{x}」解锁</t>
+          <t>挂上：{x}</t>
         </is>
       </c>
       <c r="B253" s="8" t="inlineStr">
         <is>
-          <t>通关「{x}」解锁</t>
+          <t>挂上：{x}</t>
         </is>
       </c>
       <c r="C253" s="8" t="inlineStr">
         <is>
-          <t>Clear “{x}” to unlock</t>
+          <t>Applies: {x}</t>
         </is>
       </c>
       <c r="D253" s="8" t="inlineStr">
         <is>
-          <t>Termine « {x} » pour débloquer</t>
+          <t>Applique : {x}</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" s="6" t="inlineStr">
         <is>
-          <t>挂上：{x}</t>
+          <t>难度调整：全网算力 +{n}%</t>
         </is>
       </c>
       <c r="B254" s="8" t="inlineStr">
         <is>
-          <t>挂上：{x}</t>
+          <t>难度调整：全网算力 +{n}%</t>
         </is>
       </c>
       <c r="C254" s="8" t="inlineStr">
         <is>
-          <t>Applies: {x}</t>
+          <t>Difficulty adjustment: network hash +{n}%</t>
         </is>
       </c>
       <c r="D254" s="8" t="inlineStr">
         <is>
-          <t>Applique : {x}</t>
+          <t>Ajustement de difficulté : puissance réseau +{n} %</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" s="6" t="inlineStr">
         <is>
-          <t>难度调整：全网算力 +{n}%</t>
+          <t>新知识卡</t>
         </is>
       </c>
       <c r="B255" s="8" t="inlineStr">
         <is>
-          <t>难度调整：全网算力 +{n}%</t>
+          <t>新知识卡</t>
         </is>
       </c>
       <c r="C255" s="8" t="inlineStr">
         <is>
-          <t>Difficulty adjustment: network hash +{n}%</t>
+          <t>New knowledge card</t>
         </is>
       </c>
       <c r="D255" s="8" t="inlineStr">
         <is>
-          <t>Ajustement de difficulté : puissance réseau +{n} %</t>
+          <t>Nouvelle carte savoir</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="6" t="inlineStr">
         <is>
-          <t>新知识卡</t>
+          <t>⛏ 挖矿</t>
         </is>
       </c>
       <c r="B256" s="8" t="inlineStr">
         <is>
-          <t>新知识卡</t>
+          <t>⛏ 挖矿</t>
         </is>
       </c>
       <c r="C256" s="8" t="inlineStr">
         <is>
-          <t>New knowledge card</t>
+          <t>⛏ Mining</t>
         </is>
       </c>
       <c r="D256" s="8" t="inlineStr">
         <is>
-          <t>Nouvelle carte savoir</t>
+          <t>⛏ Minage</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="6" t="inlineStr">
         <is>
-          <t>⛏ 挖矿</t>
+          <t>获得积分</t>
         </is>
       </c>
       <c r="B257" s="8" t="inlineStr">
         <is>
-          <t>⛏ 挖矿</t>
+          <t>获得积分</t>
         </is>
       </c>
       <c r="C257" s="8" t="inlineStr">
         <is>
-          <t>⛏ Mining</t>
+          <t>Points earned</t>
         </is>
       </c>
       <c r="D257" s="8" t="inlineStr">
         <is>
-          <t>⛏ Minage</t>
+          <t>Points gagnés</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="6" t="inlineStr">
         <is>
-          <t>获得积分</t>
+          <t>再点一次离开（本局进度不保存）</t>
         </is>
       </c>
       <c r="B258" s="8" t="inlineStr">
         <is>
-          <t>获得积分</t>
+          <t>再点一次离开（本局进度不保存）</t>
         </is>
       </c>
       <c r="C258" s="8" t="inlineStr">
         <is>
-          <t>Points earned</t>
+          <t>Tap again to leave (this run is not saved)</t>
         </is>
       </c>
       <c r="D258" s="8" t="inlineStr">
         <is>
-          <t>Points gagnés</t>
+          <t>Touche encore pour quitter (partie non sauvegardée)</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="6" t="inlineStr">
         <is>
-          <t>再点一次离开（本局进度不保存）</t>
+          <t>皮厚</t>
         </is>
       </c>
       <c r="B259" s="8" t="inlineStr">
         <is>
-          <t>再点一次离开（本局进度不保存）</t>
+          <t>皮厚</t>
         </is>
       </c>
       <c r="C259" s="8" t="inlineStr">
         <is>
-          <t>Tap again to leave (this run is not saved)</t>
+          <t>Tough</t>
         </is>
       </c>
       <c r="D259" s="8" t="inlineStr">
         <is>
-          <t>Touche encore pour quitter (partie non sauvegardée)</t>
+          <t>Coriace</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="6" t="inlineStr">
         <is>
-          <t>皮厚</t>
+          <t>防水</t>
         </is>
       </c>
       <c r="B260" s="8" t="inlineStr">
         <is>
-          <t>皮厚</t>
+          <t>防水</t>
         </is>
       </c>
       <c r="C260" s="8" t="inlineStr">
         <is>
-          <t>Tough</t>
+          <t>Waterproof</t>
         </is>
       </c>
       <c r="D260" s="8" t="inlineStr">
         <is>
-          <t>Coriace</t>
+          <t>Imperméable</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="6" t="inlineStr">
         <is>
-          <t>防水</t>
+          <t>跳过！</t>
         </is>
       </c>
       <c r="B261" s="8" t="inlineStr">
         <is>
-          <t>防水</t>
+          <t>跳过！</t>
         </is>
       </c>
       <c r="C261" s="8" t="inlineStr">
         <is>
-          <t>Waterproof</t>
+          <t>Hop!</t>
         </is>
       </c>
       <c r="D261" s="8" t="inlineStr">
         <is>
-          <t>Imperméable</t>
+          <t>Hop !</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="6" t="inlineStr">
         <is>
-          <t>跳过！</t>
+          <t>跑者</t>
         </is>
       </c>
       <c r="B262" s="8" t="inlineStr">
         <is>
-          <t>跳过！</t>
+          <t>跑者</t>
         </is>
       </c>
       <c r="C262" s="8" t="inlineStr">
         <is>
-          <t>Hop!</t>
+          <t>Runners</t>
         </is>
       </c>
       <c r="D262" s="8" t="inlineStr">
         <is>
-          <t>Hop !</t>
+          <t>Coureurs</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="6" t="inlineStr">
         <is>
-          <t>跑者</t>
+          <t>对策</t>
         </is>
       </c>
       <c r="B263" s="8" t="inlineStr">
         <is>
-          <t>跑者</t>
+          <t>对策</t>
         </is>
       </c>
       <c r="C263" s="8" t="inlineStr">
         <is>
-          <t>Runners</t>
+          <t>Counter</t>
         </is>
       </c>
       <c r="D263" s="8" t="inlineStr">
         <is>
-          <t>Coureurs</t>
+          <t>Parade</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="6" t="inlineStr">
         <is>
-          <t>对策</t>
+          <t>还没遇到过。</t>
         </is>
       </c>
       <c r="B264" s="8" t="inlineStr">
         <is>
-          <t>对策</t>
+          <t>还没遇到过。</t>
         </is>
       </c>
       <c r="C264" s="8" t="inlineStr">
         <is>
-          <t>Counter</t>
+          <t>Not met yet.</t>
         </is>
       </c>
       <c r="D264" s="8" t="inlineStr">
         <is>
-          <t>Parade</t>
+          <t>Pas encore croisé.</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" s="6" t="inlineStr">
         <is>
-          <t>还没遇到过。</t>
+          <t>新跑者</t>
         </is>
       </c>
       <c r="B265" s="8" t="inlineStr">
         <is>
-          <t>还没遇到过。</t>
+          <t>新跑者</t>
         </is>
       </c>
       <c r="C265" s="8" t="inlineStr">
         <is>
-          <t>Not met yet.</t>
+          <t>New runner</t>
         </is>
       </c>
       <c r="D265" s="8" t="inlineStr">
         <is>
-          <t>Pas encore croisé.</t>
+          <t>Nouveau coureur</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" s="6" t="inlineStr">
         <is>
-          <t>新跑者</t>
+          <t>对{x}无效</t>
         </is>
       </c>
       <c r="B266" s="8" t="inlineStr">
         <is>
-          <t>新跑者</t>
+          <t>对{x}无效</t>
         </is>
       </c>
       <c r="C266" s="8" t="inlineStr">
         <is>
-          <t>New runner</t>
+          <t>No effect on {x}</t>
         </is>
       </c>
       <c r="D266" s="8" t="inlineStr">
         <is>
-          <t>Nouveau coureur</t>
+          <t>Sans effet sur {x}</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="6" t="inlineStr">
         <is>
-          <t>对{x}无效</t>
+          <t>连撞 ×{n}</t>
         </is>
       </c>
       <c r="B267" s="8" t="inlineStr">
         <is>
-          <t>对{x}无效</t>
+          <t>连撞 ×{n}</t>
         </is>
       </c>
       <c r="C267" s="8" t="inlineStr">
         <is>
-          <t>No effect on {x}</t>
+          <t>Crash ×{n}</t>
         </is>
       </c>
       <c r="D267" s="8" t="inlineStr">
         <is>
-          <t>Sans effet sur {x}</t>
+          <t>Collision ×{n}</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="6" t="inlineStr">
         <is>
-          <t>连撞 ×{n}</t>
+          <t>整道铺皮！</t>
         </is>
       </c>
       <c r="B268" s="8" t="inlineStr">
         <is>
-          <t>连撞 ×{n}</t>
+          <t>整道铺皮！</t>
         </is>
       </c>
       <c r="C268" s="8" t="inlineStr">
         <is>
-          <t>Crash ×{n}</t>
+          <t>Paved with peels!</t>
         </is>
       </c>
       <c r="D268" s="8" t="inlineStr">
         <is>
-          <t>Collision ×{n}</t>
+          <t>Piste couverte !</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="6" t="inlineStr">
         <is>
-          <t>整道铺皮！</t>
+          <t>后勤补给！</t>
         </is>
       </c>
       <c r="B269" s="8" t="inlineStr">
         <is>
-          <t>整道铺皮！</t>
+          <t>后勤补给！</t>
         </is>
       </c>
       <c r="C269" s="8" t="inlineStr">
         <is>
-          <t>Paved with peels!</t>
+          <t>Supplies in!</t>
         </is>
       </c>
       <c r="D269" s="8" t="inlineStr">
         <is>
-          <t>Piste couverte !</t>
+          <t>Ravitaillement !</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="6" t="inlineStr">
         <is>
-          <t>后勤补给！</t>
+          <t>重低音 ×{n}</t>
         </is>
       </c>
       <c r="B270" s="8" t="inlineStr">
         <is>
-          <t>后勤补给！</t>
+          <t>重低音 ×{n}</t>
         </is>
       </c>
       <c r="C270" s="8" t="inlineStr">
         <is>
-          <t>Supplies in!</t>
+          <t>Bass drop ×{n}</t>
         </is>
       </c>
       <c r="D270" s="8" t="inlineStr">
         <is>
-          <t>Ravitaillement !</t>
+          <t>Basse ×{n}</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="6" t="inlineStr">
         <is>
-          <t>重低音 ×{n}</t>
+          <t>限量发售！</t>
         </is>
       </c>
       <c r="B271" s="8" t="inlineStr">
         <is>
-          <t>重低音 ×{n}</t>
+          <t>限量发售！</t>
         </is>
       </c>
       <c r="C271" s="8" t="inlineStr">
         <is>
-          <t>Bass drop ×{n}</t>
+          <t>Launch event!</t>
         </is>
       </c>
       <c r="D271" s="8" t="inlineStr">
         <is>
-          <t>Basse ×{n}</t>
+          <t>Lancement !</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="6" t="inlineStr">
         <is>
-          <t>限量发售！</t>
+          <t>投递区已设定</t>
         </is>
       </c>
       <c r="B272" s="8" t="inlineStr">
         <is>
-          <t>限量发售！</t>
+          <t>投递区已设定</t>
         </is>
       </c>
       <c r="C272" s="8" t="inlineStr">
         <is>
-          <t>Launch event!</t>
+          <t>Drop zone set</t>
         </is>
       </c>
       <c r="D272" s="8" t="inlineStr">
         <is>
-          <t>Lancement !</t>
+          <t>Zone de largage fixée</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="6" t="inlineStr">
         <is>
-          <t>投递区已设定</t>
+          <t>布阵路段已设定</t>
         </is>
       </c>
       <c r="B273" s="8" t="inlineStr">
         <is>
-          <t>投递区已设定</t>
+          <t>布阵路段已设定</t>
         </is>
       </c>
       <c r="C273" s="8" t="inlineStr">
         <is>
-          <t>Drop zone set</t>
+          <t>Trap stretch set</t>
         </is>
       </c>
       <c r="D273" s="8" t="inlineStr">
         <is>
-          <t>Zone de largage fixée</t>
+          <t>Tronçon piégé fixé</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" s="6" t="inlineStr">
         <is>
-          <t>布阵路段已设定</t>
+          <t>副路线最多 2 级</t>
         </is>
       </c>
       <c r="B274" s="8" t="inlineStr">
         <is>
-          <t>布阵路段已设定</t>
+          <t>副路线最多 2 级</t>
         </is>
       </c>
       <c r="C274" s="8" t="inlineStr">
         <is>
-          <t>Trap stretch set</t>
+          <t>Secondary path max tier 2</t>
         </is>
       </c>
       <c r="D274" s="8" t="inlineStr">
         <is>
-          <t>Tronçon piégé fixé</t>
+          <t>Voie secondaire : niveau 2 max</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="6" t="inlineStr">
         <is>
-          <t>副路线最多 2 级</t>
+          <t>6 级专精 −30%</t>
         </is>
       </c>
       <c r="B275" s="8" t="inlineStr">
         <is>
-          <t>副路线最多 2 级</t>
+          <t>6 级专精 −30%</t>
         </is>
       </c>
       <c r="C275" s="8" t="inlineStr">
         <is>
-          <t>Secondary path max tier 2</t>
+          <t>Tier-6 specialisation −30%</t>
         </is>
       </c>
       <c r="D275" s="8" t="inlineStr">
         <is>
-          <t>Voie secondaire : niveau 2 max</t>
+          <t>Spécialisation niv. 6 −30 %</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" s="6" t="inlineStr">
         <is>
-          <t>6 级专精 −30%</t>
+          <t>副</t>
         </is>
       </c>
       <c r="B276" s="8" t="inlineStr">
         <is>
-          <t>6 级专精 −30%</t>
+          <t>副</t>
         </is>
       </c>
       <c r="C276" s="8" t="inlineStr">
         <is>
-          <t>Tier-6 specialisation −30%</t>
+          <t>2nd</t>
         </is>
       </c>
       <c r="D276" s="8" t="inlineStr">
         <is>
-          <t>Spécialisation niv. 6 −30 %</t>
+          <t>2e</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="6" t="inlineStr">
         <is>
-          <t>副</t>
+          <t>副路线</t>
         </is>
       </c>
       <c r="B277" s="8" t="inlineStr">
         <is>
-          <t>副</t>
+          <t>副路线</t>
         </is>
       </c>
       <c r="C277" s="8" t="inlineStr">
         <is>
-          <t>2nd</t>
+          <t>Secondary</t>
         </is>
       </c>
       <c r="D277" s="8" t="inlineStr">
         <is>
-          <t>2e</t>
+          <t>Secondaire</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="6" t="inlineStr">
         <is>
-          <t>副路线</t>
+          <t>6 级会移除副路线，已花的 {n} GST 抵扣</t>
         </is>
       </c>
       <c r="B278" s="8" t="inlineStr">
         <is>
-          <t>副路线</t>
+          <t>6 级会移除副路线，已花的 {n} GST 抵扣</t>
         </is>
       </c>
       <c r="C278" s="8" t="inlineStr">
         <is>
-          <t>Secondary</t>
+          <t>Tier 6 removes the secondary path; the {n} GST spent on it is credited</t>
         </is>
       </c>
       <c r="D278" s="8" t="inlineStr">
         <is>
-          <t>Secondaire</t>
+          <t>Le niveau 6 retire la voie secondaire ; les {n} GST dépensés sont déduits</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" s="6" t="inlineStr">
         <is>
-          <t>6 级会移除副路线，已花的 {n} GST 抵扣</t>
+          <t>点地图上的跑道…</t>
         </is>
       </c>
       <c r="B279" s="8" t="inlineStr">
         <is>
-          <t>6 级会移除副路线，已花的 {n} GST 抵扣</t>
+          <t>点地图上的跑道…</t>
         </is>
       </c>
       <c r="C279" s="8" t="inlineStr">
         <is>
-          <t>Tier 6 removes the secondary path; the {n} GST spent on it is credited</t>
+          <t>Tap the track…</t>
         </is>
       </c>
       <c r="D279" s="8" t="inlineStr">
         <is>
-          <t>Le niveau 6 retire la voie secondaire ; les {n} GST dépensés sont déduits</t>
+          <t>Touche la piste…</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="6" t="inlineStr">
         <is>
-          <t>点地图上的跑道…</t>
+          <t>🎯 设定投递区</t>
         </is>
       </c>
       <c r="B280" s="8" t="inlineStr">
         <is>
-          <t>点地图上的跑道…</t>
+          <t>🎯 设定投递区</t>
         </is>
       </c>
       <c r="C280" s="8" t="inlineStr">
         <is>
-          <t>Tap the track…</t>
+          <t>🎯 Set drop zone</t>
         </is>
       </c>
       <c r="D280" s="8" t="inlineStr">
         <is>
-          <t>Touche la piste…</t>
+          <t>🎯 Zone de largage</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" s="6" t="inlineStr">
         <is>
-          <t>🎯 设定投递区</t>
+          <t>🎯 设定布阵路段</t>
         </is>
       </c>
       <c r="B281" s="8" t="inlineStr">
         <is>
-          <t>🎯 设定投递区</t>
+          <t>🎯 设定布阵路段</t>
         </is>
       </c>
       <c r="C281" s="8" t="inlineStr">
         <is>
-          <t>🎯 Set drop zone</t>
+          <t>🎯 Set trap stretch</t>
         </is>
       </c>
       <c r="D281" s="8" t="inlineStr">
         <is>
-          <t>🎯 Zone de largage</t>
+          <t>🎯 Tronçon à piéger</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="6" t="inlineStr">
         <is>
-          <t>🎯 设定布阵路段</t>
+          <t>两条路线可各升到 2 级；先到 3 级的是主路线，最高 5 级；6 级专精会移除副路线</t>
         </is>
       </c>
       <c r="B282" s="8" t="inlineStr">
         <is>
-          <t>🎯 设定布阵路段</t>
+          <t>两条路线可各升到 2 级；先到 3 级的是主路线，最高 5 级；6 级专精会移除副路线</t>
         </is>
       </c>
       <c r="C282" s="8" t="inlineStr">
         <is>
-          <t>🎯 Set trap stretch</t>
+          <t>Two paths can each reach tier 2; the first to tier 3 becomes main (up to 5); tier 6 specialisation removes the secondary</t>
         </is>
       </c>
       <c r="D282" s="8" t="inlineStr">
         <is>
-          <t>🎯 Tronçon à piéger</t>
+          <t>Deux voies peuvent atteindre le niveau 2 ; la première au niveau 3 devient principale (jusqu’à 5) ; la spécialisation niv. 6 retire la secondaire</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="6" t="inlineStr">
         <is>
-          <t>两条路线可各升到 2 级；先到 3 级的是主路线，最高 5 级；6 级专精会移除副路线</t>
+          <t>{x} 专精！</t>
         </is>
       </c>
       <c r="B283" s="8" t="inlineStr">
         <is>
-          <t>两条路线可各升到 2 级；先到 3 级的是主路线，最高 5 级；6 级专精会移除副路线</t>
+          <t>{x} 专精！</t>
         </is>
       </c>
       <c r="C283" s="8" t="inlineStr">
         <is>
-          <t>Two paths can each reach tier 2; the first to tier 3 becomes main (up to 5); tier 6 specialisation removes the secondary</t>
+          <t>{x} specialisation!</t>
         </is>
       </c>
       <c r="D283" s="8" t="inlineStr">
         <is>
-          <t>Deux voies peuvent atteindre le niveau 2 ; la première au niveau 3 devient principale (jusqu’à 5) ; la spécialisation niv. 6 retire la secondaire</t>
+          <t>Spécialisation : {x} !</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="6" t="inlineStr">
         <is>
-          <t>{x} 专精！</t>
+          <t>场上上限</t>
         </is>
       </c>
       <c r="B284" s="8" t="inlineStr">
         <is>
-          <t>{x} 专精！</t>
+          <t>场上上限</t>
         </is>
       </c>
       <c r="C284" s="8" t="inlineStr">
         <is>
-          <t>{x} specialisation!</t>
+          <t>Max on track</t>
         </is>
       </c>
       <c r="D284" s="8" t="inlineStr">
         <is>
-          <t>Spécialisation : {x} !</t>
+          <t>Max sur piste</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="6" t="inlineStr">
         <is>
-          <t>场上上限</t>
+          <t>每次箱数</t>
         </is>
       </c>
       <c r="B285" s="8" t="inlineStr">
         <is>
-          <t>场上上限</t>
+          <t>每次箱数</t>
         </is>
       </c>
       <c r="C285" s="8" t="inlineStr">
         <is>
-          <t>Max on track</t>
+          <t>Boxes per run</t>
         </is>
       </c>
       <c r="D285" s="8" t="inlineStr">
         <is>
-          <t>Max sur piste</t>
+          <t>Boîtes par sortie</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="6" t="inlineStr">
         <is>
-          <t>每次箱数</t>
+          <t>每次招呼</t>
         </is>
       </c>
       <c r="B286" s="8" t="inlineStr">
         <is>
-          <t>每次箱数</t>
+          <t>每次招呼</t>
         </is>
       </c>
       <c r="C286" s="8" t="inlineStr">
         <is>
-          <t>Boxes per run</t>
+          <t>Per invite</t>
         </is>
       </c>
       <c r="D286" s="8" t="inlineStr">
         <is>
-          <t>Boîtes par sortie</t>
+          <t>Par invitation</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="6" t="inlineStr">
         <is>
-          <t>每次招呼</t>
+          <t>停留</t>
         </is>
       </c>
       <c r="B287" s="8" t="inlineStr">
         <is>
-          <t>每次招呼</t>
+          <t>停留</t>
         </is>
       </c>
       <c r="C287" s="8" t="inlineStr">
         <is>
-          <t>Per invite</t>
+          <t>Stay</t>
         </is>
       </c>
       <c r="D287" s="8" t="inlineStr">
         <is>
-          <t>Par invitation</t>
+          <t>Arrêt</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="6" t="inlineStr">
         <is>
-          <t>停留</t>
+          <t>{x} 的动画 JSON 读不出来</t>
         </is>
       </c>
       <c r="B288" s="8" t="inlineStr">
         <is>
-          <t>停留</t>
+          <t>{x} 的动画 JSON 读不出来</t>
         </is>
       </c>
       <c r="C288" s="8" t="inlineStr">
         <is>
-          <t>Stay</t>
+          <t>Could not read the animation JSON for {x}</t>
         </is>
       </c>
       <c r="D288" s="8" t="inlineStr">
         <is>
-          <t>Arrêt</t>
+          <t>Impossible de lire le JSON d’animation de {x}</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="6" t="inlineStr">
         <is>
-          <t>{x} 的动画 JSON 读不出来</t>
+          <t>弹道 {x} {k}</t>
         </is>
       </c>
       <c r="B289" s="8" t="inlineStr">
         <is>
-          <t>{x} 的动画 JSON 读不出来</t>
+          <t>弹道 {x} {k}</t>
         </is>
       </c>
       <c r="C289" s="8" t="inlineStr">
         <is>
-          <t>Could not read the animation JSON for {x}</t>
+          <t>Trajectory {x} {k}</t>
         </is>
       </c>
       <c r="D289" s="8" t="inlineStr">
         <is>
-          <t>Impossible de lire le JSON d’animation de {x}</t>
+          <t>Trajectoire {x} {k}</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" s="6" t="inlineStr">
         <is>
-          <t>弹道 {x} {k}</t>
+          <t>装置 {x}：基础附加效果「{y}」写法有误，保留原效果</t>
         </is>
       </c>
       <c r="B290" s="8" t="inlineStr">
         <is>
-          <t>弹道 {x} {k}</t>
+          <t>装置 {x}：基础附加效果「{y}」写法有误，保留原效果</t>
         </is>
       </c>
       <c r="C290" s="8" t="inlineStr">
         <is>
-          <t>Trajectory {x} {k}</t>
+          <t>Device {x}: base extra effect “{y}” is malformed, kept the original</t>
         </is>
       </c>
       <c r="D290" s="8" t="inlineStr">
         <is>
-          <t>Trajectoire {x} {k}</t>
+          <t>Dispositif {x} : effet de base « {y} » mal écrit, original conservé</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" s="6" t="inlineStr">
         <is>
-          <t>装置 {x}：基础附加效果「{y}」写法有误，保留原效果</t>
+          <t>导入美术图片 / 动画（可多选）</t>
         </is>
       </c>
       <c r="B291" s="8" t="inlineStr">
         <is>
-          <t>装置 {x}：基础附加效果「{y}」写法有误，保留原效果</t>
+          <t>导入美术图片 / 动画（可多选）</t>
         </is>
       </c>
       <c r="C291" s="8" t="inlineStr">
         <is>
-          <t>Device {x}: base extra effect “{y}” is malformed, kept the original</t>
+          <t>Import art / animations (multi-select)</t>
         </is>
       </c>
       <c r="D291" s="8" t="inlineStr">
         <is>
-          <t>Dispositif {x} : effet de base « {y} » mal écrit, original conservé</t>
+          <t>Importer images / animations (plusieurs)</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" s="6" t="inlineStr">
         <is>
-          <t>导入美术图片 / 动画（可多选）</t>
+          <t>点跑道，设定投递区（Esc 取消）</t>
         </is>
       </c>
       <c r="B292" s="8" t="inlineStr">
         <is>
-          <t>导入美术图片 / 动画（可多选）</t>
+          <t>点跑道，设定投递区（Esc 取消）</t>
         </is>
       </c>
       <c r="C292" s="8" t="inlineStr">
         <is>
-          <t>Import art / animations (multi-select)</t>
+          <t>Tap the track to set the drop zone (Esc to cancel)</t>
         </is>
       </c>
       <c r="D292" s="8" t="inlineStr">
         <is>
-          <t>Importer images / animations (plusieurs)</t>
+          <t>Touche la piste pour choisir la zone de largage (Échap pour annuler)</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" s="6" t="inlineStr">
         <is>
-          <t>点跑道，设定投递区（Esc 取消）</t>
+          <t>点跑道，设定布阵路段（Esc 取消）</t>
         </is>
       </c>
       <c r="B293" s="8" t="inlineStr">
         <is>
-          <t>点跑道，设定投递区（Esc 取消）</t>
+          <t>点跑道，设定布阵路段（Esc 取消）</t>
         </is>
       </c>
       <c r="C293" s="8" t="inlineStr">
         <is>
-          <t>Tap the track to set the drop zone (Esc to cancel)</t>
+          <t>Tap the track to set the trap stretch (Esc to cancel)</t>
         </is>
       </c>
       <c r="D293" s="8" t="inlineStr">
         <is>
-          <t>Touche la piste pour choisir la zone de largage (Échap pour annuler)</t>
+          <t>Touche la piste pour choisir le tronçon à piéger (Échap pour annuler)</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" s="6" t="inlineStr">
         <is>
-          <t>点跑道，设定布阵路段（Esc 取消）</t>
+          <t>放不下</t>
         </is>
       </c>
       <c r="B294" s="8" t="inlineStr">
         <is>
-          <t>点跑道，设定布阵路段（Esc 取消）</t>
+          <t>放不下</t>
         </is>
       </c>
       <c r="C294" s="8" t="inlineStr">
         <is>
-          <t>Tap the track to set the trap stretch (Esc to cancel)</t>
+          <t>No room</t>
         </is>
       </c>
       <c r="D294" s="8" t="inlineStr">
         <is>
-          <t>Touche la piste pour choisir le tronçon à piéger (Échap pour annuler)</t>
+          <t>Pas de place</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" s="6" t="inlineStr">
         <is>
-          <t>放不下</t>
+          <t>再点一次重新开始</t>
         </is>
       </c>
       <c r="B295" s="8" t="inlineStr">
         <is>
-          <t>放不下</t>
+          <t>再点一次重新开始</t>
         </is>
       </c>
       <c r="C295" s="8" t="inlineStr">
         <is>
-          <t>No room</t>
+          <t>Tap again to restart</t>
         </is>
       </c>
       <c r="D295" s="8" t="inlineStr">
         <is>
-          <t>Pas de place</t>
+          <t>Touche encore pour recommencer</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" s="6" t="inlineStr">
         <is>
-          <t>再点一次重新开始</t>
+          <t>重开本关</t>
         </is>
       </c>
       <c r="B296" s="8" t="inlineStr">
         <is>
-          <t>再点一次重新开始</t>
+          <t>重开本关</t>
         </is>
       </c>
       <c r="C296" s="8" t="inlineStr">
         <is>
-          <t>Tap again to restart</t>
+          <t>Restart level</t>
         </is>
       </c>
       <c r="D296" s="8" t="inlineStr">
         <is>
-          <t>Touche encore pour recommencer</t>
+          <t>Rejouer le niveau</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" s="6" t="inlineStr">
         <is>
-          <t>重开本关</t>
+          <t>重新开始</t>
         </is>
       </c>
       <c r="B297" s="8" t="inlineStr">
         <is>
-          <t>重开本关</t>
+          <t>重新开始</t>
         </is>
       </c>
       <c r="C297" s="8" t="inlineStr">
         <is>
-          <t>Restart level</t>
+          <t>Restart</t>
         </is>
       </c>
       <c r="D297" s="8" t="inlineStr">
         <is>
-          <t>Rejouer le niveau</t>
+          <t>Recommencer</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" s="6" t="inlineStr">
         <is>
-          <t>重新开始</t>
+          <t>↻ 重新开始</t>
         </is>
       </c>
       <c r="B298" s="8" t="inlineStr">
         <is>
-          <t>重新开始</t>
+          <t>↻ 重新开始</t>
         </is>
       </c>
       <c r="C298" s="8" t="inlineStr">
         <is>
-          <t>Restart</t>
+          <t>↻ Restart</t>
         </is>
       </c>
       <c r="D298" s="8" t="inlineStr">
         <is>
-          <t>Recommencer</t>
+          <t>↻ Recommencer</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" s="6" t="inlineStr">
         <is>
-          <t>↻ 重新开始</t>
+          <t>点跑道外任意空地放置装置（每种装置占的格子不同），再点已放的装置升级。每个装置最多发展两条路线：都能先升到 2 级，先到 3 级的成为主路线，可升到 5 级；6 级专精会移除副路线，已花的钱抵扣。</t>
         </is>
       </c>
       <c r="B299" s="8" t="inlineStr">
         <is>
-          <t>↻ 重新开始</t>
+          <t>点跑道外任意空地放置装置（每种装置占的格子不同），再点已放的装置升级。每个装置最多发展两条路线：都能先升到 2 级，先到 3 级的成为主路线，可升到 5 级；6 级专精会移除副路线，已花的钱抵扣。</t>
         </is>
       </c>
       <c r="C299" s="8" t="inlineStr">
         <is>
-          <t>↻ Restart</t>
+          <t>Tap any free ground off the track to place a device (each device takes a different number of cells), then tap it to upgrade. Each device can grow two paths: both can reach tier 2, the first to tier 3 becomes main and goes up to 5; tier 6 specialisation removes the secondary path and credits what you spent on it.</t>
         </is>
       </c>
       <c r="D299" s="8" t="inlineStr">
         <is>
-          <t>↻ Recommencer</t>
+          <t>Touche n’importe quel terrain libre hors de la piste pour poser un dispositif (chacun occupe un nombre de cases différent), puis touche-le pour l’améliorer. Deux voies maximum : les deux peuvent atteindre le niveau 2, la première au niveau 3 devient principale jusqu’au 5 ; la spécialisation niv. 6 retire la secondaire et déduit ce que tu y as dépensé.</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" s="6" t="inlineStr">
         <is>
-          <t>点跑道外任意空地放置装置（每种装置占的格子不同），再点已放的装置升级。每个装置最多发展两条路线：都能先升到 2 级，先到 3 级的成为主路线，可升到 5 级；6 级专精会移除副路线，已花的钱抵扣。</t>
+          <t>点跑道外的空地放置装置，再点装置直接升级。</t>
         </is>
       </c>
       <c r="B300" s="8" t="inlineStr">
         <is>
-          <t>点跑道外任意空地放置装置（每种装置占的格子不同），再点已放的装置升级。每个装置最多发展两条路线：都能先升到 2 级，先到 3 级的成为主路线，可升到 5 级；6 级专精会移除副路线，已花的钱抵扣。</t>
+          <t>点跑道外的空地放置装置，再点装置直接升级。</t>
         </is>
       </c>
       <c r="C300" s="8" t="inlineStr">
         <is>
-          <t>Tap any free ground off the track to place a device (each device takes a different number of cells), then tap it to upgrade. Each device can grow two paths: both can reach tier 2, the first to tier 3 becomes main and goes up to 5; tier 6 specialisation removes the secondary path and credits what you spent on it.</t>
+          <t>Tap any free ground off the track to place a device, then tap the device to upgrade it.</t>
         </is>
       </c>
       <c r="D300" s="8" t="inlineStr">
         <is>
-          <t>Touche n’importe quel terrain libre hors de la piste pour poser un dispositif (chacun occupe un nombre de cases différent), puis touche-le pour l’améliorer. Deux voies maximum : les deux peuvent atteindre le niveau 2, la première au niveau 3 devient principale jusqu’au 5 ; la spécialisation niv. 6 retire la secondaire et déduit ce que tu y as dépensé.</t>
+          <t>Touchez un terrain libre hors de la piste pour poser un dispositif, puis touchez-le pour l’améliorer.</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" s="6" t="inlineStr">
         <is>
-          <t>点跑道外的空地放置装置，再点装置直接升级。</t>
+          <t>点跑道外的空地放置装置，再点「开始第 1 波」</t>
         </is>
       </c>
       <c r="B301" s="8" t="inlineStr">
         <is>
-          <t>点跑道外的空地放置装置，再点装置直接升级。</t>
+          <t>点跑道外的空地放置装置，再点「开始第 1 波」</t>
         </is>
       </c>
       <c r="C301" s="8" t="inlineStr">
         <is>
-          <t>Tap any free ground off the track to place a device, then tap the device to upgrade it.</t>
+          <t>Tap free ground off the track to place a device, then press “Start wave 1”</t>
         </is>
       </c>
       <c r="D301" s="8" t="inlineStr">
         <is>
-          <t>Touchez un terrain libre hors de la piste pour poser un dispositif, puis touchez-le pour l’améliorer.</t>
-        </is>
-      </c>
-    </row>
-    <row r="302">
-      <c r="A302" s="6" t="inlineStr">
-        <is>
-          <t>点跑道外的空地放置装置，再点「开始第 1 波」</t>
-        </is>
-      </c>
-      <c r="B302" s="8" t="inlineStr">
-        <is>
-          <t>点跑道外的空地放置装置，再点「开始第 1 波」</t>
-        </is>
-      </c>
-      <c r="C302" s="8" t="inlineStr">
-        <is>
-          <t>Tap free ground off the track to place a device, then press “Start wave 1”</t>
-        </is>
-      </c>
-      <c r="D302" s="8" t="inlineStr">
-        <is>
           <t>Touchez un terrain libre hors de la piste pour poser un dispositif, puis « Lancer la vague 1 »</t>
         </is>
       </c>
     </row>
-    <row r="304">
-      <c r="A304" s="10" t="inlineStr">
+    <row r="303">
+      <c r="A303" s="10" t="inlineStr">
         <is>
           <t>※ 花括号里的 {n}、{x} 等是占位符，翻译时要原样保留。</t>
         </is>
@@ -22084,7 +22115,7 @@
         <v>120</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>2.26</v>
+        <v>2.76</v>
       </c>
       <c r="H41" s="14">
         <f>G41/F41*100</f>
@@ -22124,7 +22155,7 @@
       </c>
       <c r="D42" s="9" t="inlineStr">
         <is>
-          <t>喷头加长</t>
+          <t>加长水管</t>
         </is>
       </c>
       <c r="E42" s="9" t="n">
@@ -22134,7 +22165,7 @@
         <v>180</v>
       </c>
       <c r="G42" s="9" t="n">
-        <v>2.73</v>
+        <v>3.31</v>
       </c>
       <c r="H42" s="14">
         <f>G42/F42*100</f>
@@ -22158,7 +22189,11 @@
         <f>IF(OR(K42="",L42="",L42=0),"",K42/L42)</f>
         <v/>
       </c>
-      <c r="N42" s="9" t="inlineStr"/>
+      <c r="N42" s="9" t="inlineStr">
+        <is>
+          <t>活动范围</t>
+        </is>
+      </c>
       <c r="O42" s="9">
         <f>IF(B42=0,"基准",IF(C42=6,"6 级专精：空位用完后的出路，看后期实测，不和多放基础塔比",IF(AND(N42&lt;&gt;"",I42&lt;0.85),"功能型：单看输出偏低属正常",IF(I42&gt;=0.85,"划算",IF(I42&gt;=0.65,"略亏：空位紧张时仍值得","偏亏：建议降价或加强")))))</f>
         <v/>
@@ -22188,7 +22223,7 @@
         <v>260</v>
       </c>
       <c r="G43" s="9" t="n">
-        <v>2.73</v>
+        <v>3.31</v>
       </c>
       <c r="H43" s="14">
         <f>G43/F43*100</f>
@@ -22246,7 +22281,7 @@
         <v>540</v>
       </c>
       <c r="G44" s="9" t="n">
-        <v>4.54</v>
+        <v>5.51</v>
       </c>
       <c r="H44" s="14">
         <f>G44/F44*100</f>
@@ -22300,7 +22335,7 @@
         <v>1140</v>
       </c>
       <c r="G45" s="9" t="n">
-        <v>6.49</v>
+        <v>7.87</v>
       </c>
       <c r="H45" s="14">
         <f>G45/F45*100</f>
@@ -22358,7 +22393,7 @@
         <v>2440</v>
       </c>
       <c r="G46" s="9" t="n">
-        <v>8.35</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H46" s="14">
         <f>G46/F46*100</f>
@@ -22466,7 +22501,7 @@
         <v>165</v>
       </c>
       <c r="G48" s="9" t="n">
-        <v>2.26</v>
+        <v>2.76</v>
       </c>
       <c r="H48" s="14">
         <f>G48/F48*100</f>
@@ -22524,7 +22559,7 @@
         <v>245</v>
       </c>
       <c r="G49" s="9" t="n">
-        <v>2.26</v>
+        <v>2.76</v>
       </c>
       <c r="H49" s="14">
         <f>G49/F49*100</f>
@@ -22582,7 +22617,7 @@
         <v>545</v>
       </c>
       <c r="G50" s="9" t="n">
-        <v>2.26</v>
+        <v>2.76</v>
       </c>
       <c r="H50" s="14">
         <f>G50/F50*100</f>
@@ -22640,7 +22675,7 @@
         <v>1195</v>
       </c>
       <c r="G51" s="9" t="n">
-        <v>2.26</v>
+        <v>2.76</v>
       </c>
       <c r="H51" s="14">
         <f>G51/F51*100</f>
@@ -22694,7 +22729,7 @@
         <v>2595</v>
       </c>
       <c r="G52" s="9" t="n">
-        <v>2.26</v>
+        <v>2.76</v>
       </c>
       <c r="H52" s="14">
         <f>G52/F52*100</f>
@@ -22748,7 +22783,7 @@
         <v>5995</v>
       </c>
       <c r="G53" s="9" t="n">
-        <v>11.28</v>
+        <v>13.78</v>
       </c>
       <c r="H53" s="14">
         <f>G53/F53*100</f>
@@ -22802,7 +22837,7 @@
         <v>180</v>
       </c>
       <c r="G54" s="9" t="n">
-        <v>2.88</v>
+        <v>3.38</v>
       </c>
       <c r="H54" s="14">
         <f>G54/F54*100</f>
@@ -22856,7 +22891,7 @@
         <v>290</v>
       </c>
       <c r="G55" s="9" t="n">
-        <v>5.76</v>
+        <v>6.77</v>
       </c>
       <c r="H55" s="14">
         <f>G55/F55*100</f>
@@ -22880,7 +22915,11 @@
         <f>IF(OR(K55="",L55="",L55=0),"",K55/L55)</f>
         <v/>
       </c>
-      <c r="N55" s="9" t="inlineStr"/>
+      <c r="N55" s="9" t="inlineStr">
+        <is>
+          <t>车速</t>
+        </is>
+      </c>
       <c r="O55" s="9">
         <f>IF(B55=0,"基准",IF(C55=6,"6 级专精：空位用完后的出路，看后期实测，不和多放基础塔比",IF(AND(N55&lt;&gt;"",I55&lt;0.85),"功能型：单看输出偏低属正常",IF(I55&gt;=0.85,"划算",IF(I55&gt;=0.65,"略亏：空位紧张时仍值得","偏亏：建议降价或加强")))))</f>
         <v/>
@@ -22910,7 +22949,7 @@
         <v>590</v>
       </c>
       <c r="G56" s="9" t="n">
-        <v>5.76</v>
+        <v>6.77</v>
       </c>
       <c r="H56" s="14">
         <f>G56/F56*100</f>
@@ -22968,7 +23007,7 @@
         <v>1140</v>
       </c>
       <c r="G57" s="9" t="n">
-        <v>11.94</v>
+        <v>13.51</v>
       </c>
       <c r="H57" s="14">
         <f>G57/F57*100</f>
@@ -23022,7 +23061,7 @@
         <v>2540</v>
       </c>
       <c r="G58" s="9" t="n">
-        <v>23.89</v>
+        <v>27.02</v>
       </c>
       <c r="H58" s="14">
         <f>G58/F58*100</f>
@@ -23076,7 +23115,7 @@
         <v>5940</v>
       </c>
       <c r="G59" s="9" t="n">
-        <v>71.66</v>
+        <v>81.06</v>
       </c>
       <c r="H59" s="14">
         <f>G59/F59*100</f>
@@ -27185,47 +27224,47 @@
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>洒水器</t>
+          <t>洒水车</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Sprinkler</t>
+          <t>Truck</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>Arroseur</t>
+          <t>Camion</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>洒水器</t>
+          <t>洒水车</t>
         </is>
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Sprinkler</t>
+          <t>Truck</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>Arroseur</t>
+          <t>Camion</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>持续喷水：范围内的跑者被淋湿、减速</t>
+          <t>会自己开的洒水车：在消防栓周围一圈里追着跑者开，喷到的跑者被淋湿、减速</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>Keeps spraying: runners in range get wet and slowed</t>
+          <t>Drives itself around its hydrant, chasing runners; everyone it sprays gets wet and slowed</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
         <is>
-          <t>Arrose en continu : les coureurs à portée sont mouillés et ralentis</t>
+          <t>Roule tout seul autour de sa borne à la poursuite des coureurs ; tous ceux qu’il arrose sont trempés et ralentis</t>
         </is>
       </c>
       <c r="K5" s="7" t="n">
@@ -27238,7 +27277,7 @@
         <v>1.1</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="O5" s="7" t="n">
         <v>0</v>
@@ -27268,7 +27307,7 @@
       </c>
       <c r="W5" s="7" t="inlineStr">
         <is>
-          <t>frostNeed=4; freezeCap=99</t>
+          <t>frostNeed=4; freezeCap=99; patrol=60; drive=65</t>
         </is>
       </c>
       <c r="X5" s="7" t="n">
@@ -30407,17 +30446,17 @@
       </c>
       <c r="D39" s="8" t="inlineStr">
         <is>
-          <t>喷头加长</t>
+          <t>加长水管</t>
         </is>
       </c>
       <c r="E39" s="8" t="inlineStr">
         <is>
-          <t>Longer Reach</t>
+          <t>Longer Hose</t>
         </is>
       </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
-          <t>Portée accrue</t>
+          <t>Tuyau rallongé</t>
         </is>
       </c>
       <c r="G39" s="7" t="n">
@@ -30425,22 +30464,22 @@
       </c>
       <c r="H39" s="8" t="inlineStr">
         <is>
-          <t>射程 +15</t>
+          <t>活动范围 +25，射程 +5</t>
         </is>
       </c>
       <c r="I39" s="8" t="inlineStr">
         <is>
-          <t>Range +15</t>
+          <t>Patrol +25, range +5</t>
         </is>
       </c>
       <c r="J39" s="8" t="inlineStr">
         <is>
-          <t>Portée +15</t>
+          <t>Patrouille +25, portée +5</t>
         </is>
       </c>
       <c r="K39" s="7" t="inlineStr">
         <is>
-          <t>range+=15</t>
+          <t>patrol+=25; range+=5</t>
         </is>
       </c>
       <c r="L39" s="9">
@@ -31140,22 +31179,22 @@
       </c>
       <c r="H52" s="8" t="inlineStr">
         <is>
-          <t>效果 +0.5</t>
+          <t>效果 +0.5，车速 +30%</t>
         </is>
       </c>
       <c r="I52" s="8" t="inlineStr">
         <is>
-          <t>Effect +0.5</t>
+          <t>Effect +0.5, drives 30% faster</t>
         </is>
       </c>
       <c r="J52" s="8" t="inlineStr">
         <is>
-          <t>Effet +0,5</t>
+          <t>Effet +0,5, roule 30 % plus vite</t>
         </is>
       </c>
       <c r="K52" s="7" t="inlineStr">
         <is>
-          <t>dmg+=0.5</t>
+          <t>dmg+=0.5; drive*=1.3</t>
         </is>
       </c>
       <c r="L52" s="9">

</xml_diff>